<commit_message>
User Access Maintenance FRS v1.4 on rules v2: OOTB tested against brokerverse-platform
Colour code re-done against the iNXT BrokerVerse OOTB platform (code, Feature List as
cross-check): 8 orange CRs (70.25 man-days), 5 green, 15 BRD items to deliver, 6
integration / data migration items with grey labels, 6 best-practice items in blue.
Shared helpers in colour_code.py (COLOURS, LABELS, OOTB_HEADER, legend_rows,
legend_table, add_label); e2e flow re-rendered; workbooks rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W3DAuLtsQmip7EuxjJCCtN
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-11_User_Access_Maintenance/BIBS_CR_BRD-11_Change_Request_Register_v1.1.xlsx
+++ b/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-11_User_Access_Maintenance/BIBS_CR_BRD-11_Change_Request_Register_v1.1.xlsx
@@ -16,11 +16,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'README'!$A$4:$D$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'README'!$A$4:$D$44</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'README'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'How to use'!$A$4:$D$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'How to use'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Register'!$A$4:$U$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Register'!$A$4:$W$20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Register'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Impact assessment form'!$A$12:$C$25</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Impact assessment form'!$12:$12</definedName>
@@ -939,11 +939,11 @@
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>Change requests known at v1.4 (status Candidate - for decision, effort in the CR Effort Estimate), the earlier candidates closed as BRD requirements or offered as standard, and new requests</t>
+          <t>Change requests known at v1.4 (status Candidate - for decision, effort in the CR Effort Estimate), the earlier candidates closed as BRD requirements, integration scope or offered by iNXT BrokerVerse OOTB (brokerverse-platform), and new requests</t>
         </is>
       </c>
       <c r="D22" s="12" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="23">
@@ -1035,7 +1035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>Change request (orange) / offered as standard (green) / BRD requirement (black)</t>
+          <t>Change request (orange) / offered by iNXT BrokerVerse OOTB (green) / BRD requirement (black) / integration or data migration scope (grey)</t>
         </is>
       </c>
       <c r="D10" s="14" t="inlineStr"/>
@@ -1184,12 +1184,12 @@
       </c>
       <c r="B11" s="20" t="inlineStr">
         <is>
-          <t>Date raised</t>
+          <t>Feature List ID / OOTB status</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>dd-Mmm-yyyy</t>
+          <t>Row of the Feature List vs OOTB workbook and its OOTB platform status</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr"/>
@@ -1202,12 +1202,12 @@
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>Raised by</t>
+          <t>Already in BIBS?</t>
         </is>
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>Name and role</t>
+          <t>Already available for BDOI in the BIBS system (still a change request when orange)</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr"/>
@@ -1220,12 +1220,12 @@
       </c>
       <c r="B13" s="20" t="inlineStr">
         <is>
-          <t>BRD ID</t>
+          <t>Date raised</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>BRD requirement</t>
+          <t>dd-Mmm-yyyy</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr"/>
@@ -1238,12 +1238,12 @@
       </c>
       <c r="B14" s="21" t="inlineStr">
         <is>
-          <t>FRS reference</t>
+          <t>Raised by</t>
         </is>
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
-          <t>FR item or annex</t>
+          <t>Name and role</t>
         </is>
       </c>
       <c r="D14" s="14" t="inlineStr"/>
@@ -1256,12 +1256,12 @@
       </c>
       <c r="B15" s="20" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>BRD ID</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>The change</t>
+          <t>BRD requirement</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr"/>
@@ -1274,12 +1274,12 @@
       </c>
       <c r="B16" s="21" t="inlineStr">
         <is>
-          <t>Reason</t>
+          <t>FRS reference</t>
         </is>
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>Why</t>
+          <t>FR item or annex</t>
         </is>
       </c>
       <c r="D16" s="14" t="inlineStr"/>
@@ -1292,19 +1292,15 @@
       </c>
       <c r="B17" s="20" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>Kind of change</t>
-        </is>
-      </c>
-      <c r="D17" s="12" t="inlineStr">
-        <is>
-          <t>Beyond the BRD, Added by BDOI's FRS, Proposal for best practice, Correction</t>
-        </is>
-      </c>
+          <t>The change</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
@@ -1314,10 +1310,14 @@
       </c>
       <c r="B18" s="21" t="inlineStr">
         <is>
-          <t>Impact on scope</t>
-        </is>
-      </c>
-      <c r="C18" s="14" t="inlineStr"/>
+          <t>Reason</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
       <c r="D18" s="14" t="inlineStr"/>
     </row>
     <row r="19">
@@ -1328,11 +1328,19 @@
       </c>
       <c r="B19" s="20" t="inlineStr">
         <is>
-          <t>Impact on schedule</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="inlineStr"/>
-      <c r="D19" s="12" t="inlineStr"/>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>Kind of change</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>Beyond the BRD, Added by BDOI's FRS, Proposal for best practice, Correction</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
@@ -1342,7 +1350,7 @@
       </c>
       <c r="B20" s="21" t="inlineStr">
         <is>
-          <t>Impact on cost</t>
+          <t>Impact on scope</t>
         </is>
       </c>
       <c r="C20" s="14" t="inlineStr"/>
@@ -1356,7 +1364,7 @@
       </c>
       <c r="B21" s="20" t="inlineStr">
         <is>
-          <t>Impact on other BRDs</t>
+          <t>Impact on schedule</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr"/>
@@ -1370,7 +1378,7 @@
       </c>
       <c r="B22" s="21" t="inlineStr">
         <is>
-          <t>Impact on tests</t>
+          <t>Impact on cost</t>
         </is>
       </c>
       <c r="C22" s="14" t="inlineStr"/>
@@ -1384,15 +1392,11 @@
       </c>
       <c r="B23" s="20" t="inlineStr">
         <is>
-          <t>Priority</t>
+          <t>Impact on other BRDs</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr"/>
-      <c r="D23" s="12" t="inlineStr">
-        <is>
-          <t>High, Medium, Low</t>
-        </is>
-      </c>
+      <c r="D23" s="12" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
@@ -1402,15 +1406,11 @@
       </c>
       <c r="B24" s="21" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Impact on tests</t>
         </is>
       </c>
       <c r="C24" s="14" t="inlineStr"/>
-      <c r="D24" s="14" t="inlineStr">
-        <is>
-          <t>Candidate - for decision, Raised, Assessed, Approved, Rejected, Scheduled, In test, Closed</t>
-        </is>
-      </c>
+      <c r="D24" s="14" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
@@ -1420,15 +1420,15 @@
       </c>
       <c r="B25" s="20" t="inlineStr">
         <is>
-          <t>Decision</t>
-        </is>
-      </c>
-      <c r="C25" s="12" t="inlineStr">
-        <is>
-          <t>Decision of the approvers</t>
-        </is>
-      </c>
-      <c r="D25" s="12" t="inlineStr"/>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr"/>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>High, Medium, Low</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
@@ -1438,11 +1438,15 @@
       </c>
       <c r="B26" s="21" t="inlineStr">
         <is>
-          <t>Approved by</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="C26" s="14" t="inlineStr"/>
-      <c r="D26" s="14" t="inlineStr"/>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>Candidate - for decision, Raised, Assessed, Approved, Rejected, Scheduled, In test, Closed</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="12" t="inlineStr">
@@ -1452,10 +1456,14 @@
       </c>
       <c r="B27" s="20" t="inlineStr">
         <is>
-          <t>Decision date</t>
-        </is>
-      </c>
-      <c r="C27" s="12" t="inlineStr"/>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>Decision of the approvers</t>
+        </is>
+      </c>
       <c r="D27" s="12" t="inlineStr"/>
     </row>
     <row r="28">
@@ -1466,7 +1474,7 @@
       </c>
       <c r="B28" s="21" t="inlineStr">
         <is>
-          <t>Target drop</t>
+          <t>Approved by</t>
         </is>
       </c>
       <c r="C28" s="14" t="inlineStr"/>
@@ -1480,48 +1488,40 @@
       </c>
       <c r="B29" s="20" t="inlineStr">
         <is>
-          <t>Linked test cases</t>
-        </is>
-      </c>
-      <c r="C29" s="12" t="inlineStr">
-        <is>
-          <t>Test cases of the Test Cases and Traceability workbook</t>
-        </is>
-      </c>
+          <t>Decision date</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr"/>
       <c r="D29" s="12" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>Impact assessment form</t>
+          <t>Register</t>
         </is>
       </c>
       <c r="B30" s="21" t="inlineStr">
         <is>
-          <t>Field</t>
-        </is>
-      </c>
-      <c r="C30" s="14" t="inlineStr">
-        <is>
-          <t>Part of the assessment</t>
-        </is>
-      </c>
+          <t>Target drop</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="inlineStr"/>
       <c r="D30" s="14" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
         <is>
-          <t>Impact assessment form</t>
+          <t>Register</t>
         </is>
       </c>
       <c r="B31" s="20" t="inlineStr">
         <is>
-          <t>Assessment</t>
+          <t>Linked test cases</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
-          <t>Filled in by the project</t>
+          <t>Test cases of the Test Cases and Traceability workbook</t>
         </is>
       </c>
       <c r="D31" s="12" t="inlineStr"/>
@@ -1534,12 +1534,12 @@
       </c>
       <c r="B32" s="21" t="inlineStr">
         <is>
-          <t>Assessed by</t>
+          <t>Field</t>
         </is>
       </c>
       <c r="C32" s="14" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Part of the assessment</t>
         </is>
       </c>
       <c r="D32" s="14" t="inlineStr"/>
@@ -1547,17 +1547,17 @@
     <row r="33">
       <c r="A33" s="12" t="inlineStr">
         <is>
-          <t>Decisions log</t>
+          <t>Impact assessment form</t>
         </is>
       </c>
       <c r="B33" s="20" t="inlineStr">
         <is>
-          <t>Annex Q No.</t>
+          <t>Assessment</t>
         </is>
       </c>
       <c r="C33" s="12" t="inlineStr">
         <is>
-          <t>Row of Annex Q of the FRS v1.4</t>
+          <t>Filled in by the project</t>
         </is>
       </c>
       <c r="D33" s="12" t="inlineStr"/>
@@ -1565,15 +1565,19 @@
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
-          <t>Decisions log</t>
+          <t>Impact assessment form</t>
         </is>
       </c>
       <c r="B34" s="21" t="inlineStr">
         <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C34" s="14" t="inlineStr"/>
+          <t>Assessed by</t>
+        </is>
+      </c>
+      <c r="C34" s="14" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
       <c r="D34" s="14" t="inlineStr"/>
     </row>
     <row r="35">
@@ -1584,10 +1588,14 @@
       </c>
       <c r="B35" s="20" t="inlineStr">
         <is>
-          <t>Topic</t>
-        </is>
-      </c>
-      <c r="C35" s="12" t="inlineStr"/>
+          <t>Annex Q No.</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>Row of Annex Q of the FRS v1.4</t>
+        </is>
+      </c>
       <c r="D35" s="12" t="inlineStr"/>
     </row>
     <row r="36">
@@ -1598,7 +1606,7 @@
       </c>
       <c r="B36" s="21" t="inlineStr">
         <is>
-          <t>Proposed in the FRS</t>
+          <t>Section</t>
         </is>
       </c>
       <c r="C36" s="14" t="inlineStr"/>
@@ -1612,7 +1620,7 @@
       </c>
       <c r="B37" s="20" t="inlineStr">
         <is>
-          <t>Decision by</t>
+          <t>Topic</t>
         </is>
       </c>
       <c r="C37" s="12" t="inlineStr"/>
@@ -1626,14 +1634,10 @@
       </c>
       <c r="B38" s="21" t="inlineStr">
         <is>
-          <t>Decision</t>
-        </is>
-      </c>
-      <c r="C38" s="14" t="inlineStr">
-        <is>
-          <t>Adopt proposal / Keep BDOI text / Other</t>
-        </is>
-      </c>
+          <t>Proposed in the FRS</t>
+        </is>
+      </c>
+      <c r="C38" s="14" t="inlineStr"/>
       <c r="D38" s="14" t="inlineStr"/>
     </row>
     <row r="39">
@@ -1644,7 +1648,7 @@
       </c>
       <c r="B39" s="20" t="inlineStr">
         <is>
-          <t>Decided by (name)</t>
+          <t>Decision by</t>
         </is>
       </c>
       <c r="C39" s="12" t="inlineStr"/>
@@ -1658,10 +1662,14 @@
       </c>
       <c r="B40" s="21" t="inlineStr">
         <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="C40" s="14" t="inlineStr"/>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="C40" s="14" t="inlineStr">
+        <is>
+          <t>Adopt proposal / Keep BDOI text / Other</t>
+        </is>
+      </c>
       <c r="D40" s="14" t="inlineStr"/>
     </row>
     <row r="41">
@@ -1672,7 +1680,7 @@
       </c>
       <c r="B41" s="20" t="inlineStr">
         <is>
-          <t>CR No. (if a change follows)</t>
+          <t>Decided by (name)</t>
         </is>
       </c>
       <c r="C41" s="12" t="inlineStr"/>
@@ -1686,18 +1694,46 @@
       </c>
       <c r="B42" s="21" t="inlineStr">
         <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C42" s="14" t="inlineStr"/>
+      <c r="D42" s="14" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="12" t="inlineStr">
+        <is>
+          <t>Decisions log</t>
+        </is>
+      </c>
+      <c r="B43" s="20" t="inlineStr">
+        <is>
+          <t>CR No. (if a change follows)</t>
+        </is>
+      </c>
+      <c r="C43" s="12" t="inlineStr"/>
+      <c r="D43" s="12" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="14" t="inlineStr">
+        <is>
+          <t>Decisions log</t>
+        </is>
+      </c>
+      <c r="B44" s="21" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C42" s="14" t="inlineStr"/>
-      <c r="D42" s="14" t="inlineStr">
+      <c r="C44" s="14" t="inlineStr"/>
+      <c r="D44" s="14" t="inlineStr">
         <is>
           <t>Open, Decided, Withdrawn</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:D42"/>
+  <autoFilter ref="A4:D44"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>
@@ -1931,30 +1967,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U19"/>
+  <dimension ref="A1:W20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="46" customWidth="1" min="7" max="7"/>
-    <col width="36" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="24" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="30" customWidth="1" min="21" max="21"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="46" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="24" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="30" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -1967,7 +2005,7 @@
     <row r="2">
       <c r="A2" s="22" t="inlineStr">
         <is>
-          <t>Change requests known at v1.4 (status Candidate - for decision, effort in the CR Effort Estimate), the earlier candidates closed as BRD requirements or offered as standard, and new requests</t>
+          <t>Change requests known at v1.4 (status Candidate - for decision, effort in the CR Effort Estimate), the earlier candidates closed as BRD requirements, integration scope or offered by iNXT BrokerVerse OOTB (brokerverse-platform), and new requests</t>
         </is>
       </c>
     </row>
@@ -1993,6 +2031,8 @@
       <c r="S3" s="23" t="n"/>
       <c r="T3" s="23" t="n"/>
       <c r="U3" s="23" t="n"/>
+      <c r="V3" s="23" t="n"/>
+      <c r="W3" s="23" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="24" t="inlineStr">
@@ -2007,95 +2047,105 @@
       </c>
       <c r="C4" s="24" t="inlineStr">
         <is>
+          <t>Feature List ID / OOTB status</t>
+        </is>
+      </c>
+      <c r="D4" s="24" t="inlineStr">
+        <is>
+          <t>Already in BIBS?</t>
+        </is>
+      </c>
+      <c r="E4" s="24" t="inlineStr">
+        <is>
           <t>Date raised</t>
         </is>
       </c>
-      <c r="D4" s="24" t="inlineStr">
+      <c r="F4" s="24" t="inlineStr">
         <is>
           <t>Raised by</t>
         </is>
       </c>
-      <c r="E4" s="24" t="inlineStr">
+      <c r="G4" s="24" t="inlineStr">
         <is>
           <t>BRD ID</t>
         </is>
       </c>
-      <c r="F4" s="24" t="inlineStr">
+      <c r="H4" s="24" t="inlineStr">
         <is>
           <t>FRS reference</t>
         </is>
       </c>
-      <c r="G4" s="24" t="inlineStr">
+      <c r="I4" s="24" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="H4" s="24" t="inlineStr">
+      <c r="J4" s="24" t="inlineStr">
         <is>
           <t>Reason</t>
         </is>
       </c>
-      <c r="I4" s="24" t="inlineStr">
+      <c r="K4" s="24" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="J4" s="24" t="inlineStr">
+      <c r="L4" s="24" t="inlineStr">
         <is>
           <t>Impact on scope</t>
         </is>
       </c>
-      <c r="K4" s="24" t="inlineStr">
+      <c r="M4" s="24" t="inlineStr">
         <is>
           <t>Impact on schedule</t>
         </is>
       </c>
-      <c r="L4" s="24" t="inlineStr">
+      <c r="N4" s="24" t="inlineStr">
         <is>
           <t>Impact on cost</t>
         </is>
       </c>
-      <c r="M4" s="24" t="inlineStr">
+      <c r="O4" s="24" t="inlineStr">
         <is>
           <t>Impact on other BRDs</t>
         </is>
       </c>
-      <c r="N4" s="24" t="inlineStr">
+      <c r="P4" s="24" t="inlineStr">
         <is>
           <t>Impact on tests</t>
         </is>
       </c>
-      <c r="O4" s="24" t="inlineStr">
+      <c r="Q4" s="24" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="P4" s="24" t="inlineStr">
+      <c r="R4" s="24" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="Q4" s="24" t="inlineStr">
+      <c r="S4" s="24" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="R4" s="24" t="inlineStr">
+      <c r="T4" s="24" t="inlineStr">
         <is>
           <t>Approved by</t>
         </is>
       </c>
-      <c r="S4" s="24" t="inlineStr">
+      <c r="U4" s="24" t="inlineStr">
         <is>
           <t>Decision date</t>
         </is>
       </c>
-      <c r="T4" s="24" t="inlineStr">
+      <c r="V4" s="24" t="inlineStr">
         <is>
           <t>Target drop</t>
         </is>
       </c>
-      <c r="U4" s="24" t="inlineStr">
+      <c r="W4" s="24" t="inlineStr">
         <is>
           <t>Linked test cases</t>
         </is>
@@ -2109,96 +2159,106 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Offered as standard (OB-UA-01, green in the FRS)</t>
+          <t>Offered by iNXT BrokerVerse OOTB (OB-UA-01, green in the FRS)</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
+          <t>UAM-018 Segregation of duties rules: Available</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
           <t>09-Oct-2026</t>
         </is>
       </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="F5" s="12" t="inlineStr">
         <is>
           <t>iorta TechNXT Project Team</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
+      <c r="G5" s="12" t="inlineStr">
         <is>
           <t>BRD NFR p.17 (11)</t>
         </is>
       </c>
-      <c r="F5" s="12" t="inlineStr">
+      <c r="H5" s="12" t="inlineStr">
         <is>
           <t>FRUM.012.01</t>
         </is>
       </c>
-      <c r="G5" s="12" t="inlineStr">
+      <c r="I5" s="12" t="inlineStr">
         <is>
           <t>Separation-of-duties rules: Pairs of group profiles one user may not hold, kept by the Business Administrator and authorised by Information Security; checked on every request.</t>
         </is>
       </c>
-      <c r="H5" s="12" t="inlineStr">
+      <c r="J5" s="12" t="inlineStr">
         <is>
           <t>The BRD asks to monitor and escalate privilege changes; the rules are a means proposed by the project.</t>
         </is>
       </c>
-      <c r="I5" s="12" t="inlineStr">
+      <c r="K5" s="12" t="inlineStr">
         <is>
           <t>Beyond the BRD</t>
         </is>
       </c>
-      <c r="J5" s="12" t="inlineStr">
+      <c r="L5" s="12" t="inlineStr">
         <is>
           <t>None (available)</t>
         </is>
       </c>
-      <c r="K5" s="12" t="inlineStr">
+      <c r="M5" s="12" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="L5" s="12" t="inlineStr">
+      <c r="N5" s="12" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="M5" s="12" t="inlineStr">
+      <c r="O5" s="12" t="inlineStr">
         <is>
           <t>All modules (roles)</t>
         </is>
       </c>
-      <c r="N5" s="12" t="inlineStr">
+      <c r="P5" s="12" t="inlineStr">
         <is>
           <t>FRUM.012.01 cases</t>
         </is>
       </c>
-      <c r="O5" s="12" t="inlineStr">
+      <c r="Q5" s="12" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="P5" s="25" t="inlineStr">
+      <c r="R5" s="25" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="Q5" s="12" t="inlineStr">
-        <is>
-          <t>Not a change request (review of 11-Oct-2026): Offered as standard (separation-of-duties rules, authorised by Information Security); extends the segregation-of-duties principle of the Operations addendum. No change request, no cost.</t>
-        </is>
-      </c>
-      <c r="R5" s="12" t="inlineStr">
+      <c r="S5" s="12" t="inlineStr">
+        <is>
+          <t>Not a change request (review of 11-Oct-2026): Offered by the iNXT BrokerVerse OOTB platform (separation-of-duties rules on pairs of roles, block or warn); extends the segregation-of-duties principle of the Operations addendum. No change request, no cost.</t>
+        </is>
+      </c>
+      <c r="T5" s="12" t="inlineStr">
         <is>
           <t>iorta TechNXT Project Team (for BDOI confirmation)</t>
         </is>
       </c>
-      <c r="S5" s="12" t="inlineStr">
+      <c r="U5" s="12" t="inlineStr">
         <is>
           <t>11-Oct-2026</t>
         </is>
       </c>
-      <c r="T5" s="12" t="inlineStr"/>
-      <c r="U5" s="12" t="inlineStr">
+      <c r="V5" s="12" t="inlineStr"/>
+      <c r="W5" s="12" t="inlineStr">
         <is>
           <t>TC-FRUM-012.01-AC01, TC-FRUM-012.01-AC02, TC-UA-053.1-01, TC-UA-053.2-01, TC-UA-053.2-02</t>
         </is>
@@ -2212,96 +2272,106 @@
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>Offered as standard (OB-UA-02, green in the FRS)</t>
+          <t>Offered by iNXT BrokerVerse OOTB (OB-UA-02, green in the FRS)</t>
         </is>
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
+          <t>UAM-028 Dormant account deactivation: Available</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
           <t>09-Oct-2026</t>
         </is>
       </c>
-      <c r="D6" s="12" t="inlineStr">
+      <c r="F6" s="12" t="inlineStr">
         <is>
           <t>iorta TechNXT Project Team</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
+      <c r="G6" s="12" t="inlineStr">
         <is>
           <t>BRD NFR p.13 (1.e)</t>
         </is>
       </c>
-      <c r="F6" s="12" t="inlineStr">
+      <c r="H6" s="12" t="inlineStr">
         <is>
           <t>FRUM.003.04</t>
         </is>
       </c>
-      <c r="G6" s="12" t="inlineStr">
+      <c r="I6" s="12" t="inlineStr">
         <is>
           <t>Dormant-user deactivation: Users without a sign-in for 90 days deactivated by a daily run, with a notice 7 days before.</t>
         </is>
       </c>
-      <c r="H6" s="12" t="inlineStr">
+      <c r="J6" s="12" t="inlineStr">
         <is>
           <t>Information Security practice; not in the BRD text.</t>
         </is>
       </c>
-      <c r="I6" s="12" t="inlineStr">
+      <c r="K6" s="12" t="inlineStr">
         <is>
           <t>Beyond the BRD</t>
         </is>
       </c>
-      <c r="J6" s="12" t="inlineStr">
+      <c r="L6" s="12" t="inlineStr">
         <is>
           <t>None (available)</t>
         </is>
       </c>
-      <c r="K6" s="12" t="inlineStr">
+      <c r="M6" s="12" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="L6" s="12" t="inlineStr">
+      <c r="N6" s="12" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="M6" s="12" t="inlineStr">
+      <c r="O6" s="12" t="inlineStr">
         <is>
           <t>All users</t>
         </is>
       </c>
-      <c r="N6" s="12" t="inlineStr">
+      <c r="P6" s="12" t="inlineStr">
         <is>
           <t>FRUM.003.04 cases</t>
         </is>
       </c>
-      <c r="O6" s="12" t="inlineStr">
+      <c r="Q6" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="P6" s="25" t="inlineStr">
+      <c r="R6" s="25" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="Q6" s="12" t="inlineStr">
-        <is>
-          <t>Not a change request (review of 11-Oct-2026): Offered as standard (dormant-user run, setting of 90 days and notice of 7 days). No change request, no cost.</t>
-        </is>
-      </c>
-      <c r="R6" s="12" t="inlineStr">
+      <c r="S6" s="12" t="inlineStr">
+        <is>
+          <t>Not a change request (review of 11-Oct-2026): Offered by the iNXT BrokerVerse OOTB platform (daily run deactivating accounts without a sign-in for 90 days, setting). No change request, no cost.</t>
+        </is>
+      </c>
+      <c r="T6" s="12" t="inlineStr">
         <is>
           <t>iorta TechNXT Project Team (for BDOI confirmation)</t>
         </is>
       </c>
-      <c r="S6" s="12" t="inlineStr">
+      <c r="U6" s="12" t="inlineStr">
         <is>
           <t>11-Oct-2026</t>
         </is>
       </c>
-      <c r="T6" s="12" t="inlineStr"/>
-      <c r="U6" s="12" t="inlineStr">
+      <c r="V6" s="12" t="inlineStr"/>
+      <c r="W6" s="12" t="inlineStr">
         <is>
           <t>TC-FRUM-003.04-AC01, TC-FRUM-003.04-AC02, TC-FRUM-003.04-AC03, TC-UA-006.1-01, TC-UA-006.2-01</t>
         </is>
@@ -2315,96 +2385,94 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Offered as standard (OB-UA-03, green in the FRS)</t>
+          <t>Change request (orange in the FRS)</t>
         </is>
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
+          <t>No feature row (related UAM-007 two-factor authentication: Available)</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
           <t>09-Oct-2026</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
+      <c r="F7" s="12" t="inlineStr">
         <is>
           <t>iorta TechNXT Project Team</t>
         </is>
       </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>BRD 4.001.1</t>
-        </is>
-      </c>
-      <c r="F7" s="12" t="inlineStr">
-        <is>
-          <t>FRUM.001.06</t>
-        </is>
-      </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
-          <t>Break-glass administrators: Two named System Administrator accounts with a local password and second factor when the sign-in is through EIAM; each sign-in alerted to Information Security.</t>
+          <t>Not in BRD</t>
         </is>
       </c>
       <c r="H7" s="12" t="inlineStr">
         <is>
-          <t>BDOI's FRS requires the Enterprise SSO for every sign-in; the system must stay manageable when EIAM is down.</t>
+          <t>FRUM.001.06; Annex N.4, Annex Q.5</t>
         </is>
       </c>
       <c r="I7" s="12" t="inlineStr">
         <is>
+          <t>Break-glass administrators: Two named System Administrator accounts with a local password and second factor while every other user signs in through EIAM; the sign-in method recorded; a notice and e-mail to Information Security at each break-glass sign-in; the setting of the alert addresses.</t>
+        </is>
+      </c>
+      <c r="J7" s="12" t="inlineStr">
+        <is>
+          <t>BDOI's FRS signs every user in through EIAM; two named administrator accounts must still get in when EIAM is down, with each such sign-in alerted to Information Security. The OOTB platform has local accounts only and no break-glass accounts or alert.</t>
+        </is>
+      </c>
+      <c r="K7" s="12" t="inlineStr">
+        <is>
           <t>Beyond the BRD</t>
         </is>
       </c>
-      <c r="J7" s="12" t="inlineStr">
+      <c r="L7" s="12" t="inlineStr">
         <is>
           <t>Alert to Information Security to add</t>
         </is>
       </c>
-      <c r="K7" s="12" t="inlineStr">
-        <is>
-          <t>Small</t>
-        </is>
-      </c>
-      <c r="L7" s="12" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="M7" s="12" t="inlineStr">
         <is>
+          <t>Medium complexity</t>
+        </is>
+      </c>
+      <c r="N7" s="12" t="inlineStr">
+        <is>
+          <t>6 man-days (CR Effort Estimate)</t>
+        </is>
+      </c>
+      <c r="O7" s="12" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N7" s="12" t="inlineStr">
+      <c r="P7" s="12" t="inlineStr">
         <is>
           <t>FRUM.001.06 cases</t>
         </is>
       </c>
-      <c r="O7" s="12" t="inlineStr">
+      <c r="Q7" s="12" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="P7" s="25" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="Q7" s="12" t="inlineStr">
-        <is>
-          <t>Not a change request (review of 11-Oct-2026): Offered as standard (two break-glass administrators, sign-in alerted to Information Security). No change request, no cost.</t>
-        </is>
-      </c>
-      <c r="R7" s="12" t="inlineStr">
-        <is>
-          <t>iorta TechNXT Project Team (for BDOI confirmation)</t>
-        </is>
-      </c>
-      <c r="S7" s="12" t="inlineStr">
-        <is>
-          <t>11-Oct-2026</t>
-        </is>
-      </c>
+      <c r="R7" s="25" t="inlineStr">
+        <is>
+          <t>Candidate - for decision</t>
+        </is>
+      </c>
+      <c r="S7" s="12" t="inlineStr"/>
       <c r="T7" s="12" t="inlineStr"/>
-      <c r="U7" s="12" t="inlineStr">
+      <c r="U7" s="12" t="inlineStr"/>
+      <c r="V7" s="12" t="inlineStr"/>
+      <c r="W7" s="12" t="inlineStr">
         <is>
           <t>TC-FRUM-001.06-AC01, TC-FRUM-001.06-AC02, TC-FRUM-001.06-AC03, TC-UA-003.1-01, TC-UA-003.2-01</t>
         </is>
@@ -2423,91 +2491,101 @@
       </c>
       <c r="C8" s="12" t="inlineStr">
         <is>
+          <t>UAM-003 Inactivity warning and automatic sign-out: Partial</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
           <t>09-Oct-2026</t>
         </is>
       </c>
-      <c r="D8" s="12" t="inlineStr">
+      <c r="F8" s="12" t="inlineStr">
         <is>
           <t>iorta TechNXT Project Team</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="G8" s="12" t="inlineStr">
         <is>
           <t>User Access Maintenance BRD 1.001.1.3, 2.001.1.3, 3.001.1.3, 4.001.1.3</t>
         </is>
       </c>
-      <c r="F8" s="12" t="inlineStr">
+      <c r="H8" s="12" t="inlineStr">
         <is>
           <t>FRUM.001.04</t>
         </is>
       </c>
-      <c r="G8" s="12" t="inlineStr">
+      <c r="I8" s="12" t="inlineStr">
         <is>
           <t>Warning before the fixed end of a session: Warning 30 minutes before the fixed end of a session, besides the inactivity time-out.</t>
         </is>
       </c>
-      <c r="H8" s="12" t="inlineStr">
+      <c r="J8" s="12" t="inlineStr">
         <is>
           <t>BRD reads 'warning prior to system triggered log out'; BDOI's FRS gives a time-out message instead (Annex Q, C07).</t>
         </is>
       </c>
-      <c r="I8" s="12" t="inlineStr">
+      <c r="K8" s="12" t="inlineStr">
         <is>
           <t>Correction</t>
         </is>
       </c>
-      <c r="J8" s="12" t="inlineStr">
+      <c r="L8" s="12" t="inlineStr">
         <is>
           <t>None (available)</t>
         </is>
       </c>
-      <c r="K8" s="12" t="inlineStr">
+      <c r="M8" s="12" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="L8" s="12" t="inlineStr">
+      <c r="N8" s="12" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="M8" s="12" t="inlineStr">
+      <c r="O8" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N8" s="12" t="inlineStr">
+      <c r="P8" s="12" t="inlineStr">
         <is>
           <t>FRUM.001.04 cases</t>
         </is>
       </c>
-      <c r="O8" s="12" t="inlineStr">
+      <c r="Q8" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="P8" s="25" t="inlineStr">
+      <c r="R8" s="25" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="Q8" s="12" t="inlineStr">
-        <is>
-          <t>Not a change request (review of 11-Oct-2026): Already a BRD requirement: User Access Maintenance BRD 1.001.1.3, 2.001.1.3, 3.001.1.3, 4.001.1.3 (warning prior to system triggered log out). Offered as standard.</t>
-        </is>
-      </c>
-      <c r="R8" s="12" t="inlineStr">
+      <c r="S8" s="12" t="inlineStr">
+        <is>
+          <t>Not a change request (review of 11-Oct-2026): Already a BRD requirement: User Access Maintenance BRD 1.001.1.3, 2.001.1.3, 3.001.1.3, 4.001.1.3 (warning prior to system triggered log out). The OOTB platform warns one minute before the sign-out only; the warning at 15 minutes is in scope (BRD-UA-03, Annex AA.4).</t>
+        </is>
+      </c>
+      <c r="T8" s="12" t="inlineStr">
         <is>
           <t>iorta TechNXT Project Team (for BDOI confirmation)</t>
         </is>
       </c>
-      <c r="S8" s="12" t="inlineStr">
+      <c r="U8" s="12" t="inlineStr">
         <is>
           <t>11-Oct-2026</t>
         </is>
       </c>
-      <c r="T8" s="12" t="inlineStr"/>
-      <c r="U8" s="12" t="inlineStr">
+      <c r="V8" s="12" t="inlineStr"/>
+      <c r="W8" s="12" t="inlineStr">
         <is>
           <t>TC-FRUM-001.04-AC01, TC-FRUM-001.04-AC02, TC-FRUM-001.04-AC03, TC-UA-002.1-01, TC-UA-002.1-02</t>
         </is>
@@ -2521,96 +2599,106 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Offered as standard (OB-UA-04, green in the FRS)</t>
+          <t>Integration scope (IS-UA-01, grey label in the FRS)</t>
         </is>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
+          <t>UAM-011 Directory / LDAP authentication: Not available</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
           <t>09-Oct-2026</t>
         </is>
       </c>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="F9" s="12" t="inlineStr">
         <is>
           <t>iorta TechNXT Project Team</t>
         </is>
       </c>
-      <c r="E9" s="12" t="inlineStr">
+      <c r="G9" s="12" t="inlineStr">
         <is>
           <t>BRD p.5-6</t>
         </is>
       </c>
-      <c r="F9" s="12" t="inlineStr">
+      <c r="H9" s="12" t="inlineStr">
         <is>
           <t>FRUM.002.02</t>
         </is>
       </c>
-      <c r="G9" s="12" t="inlineStr">
+      <c r="I9" s="12" t="inlineStr">
         <is>
           <t>Synchronisation of user details and status from the Enterprise SSO / UIDM-ISC: User details and status received from UIDM-ISC with the UIDM request number, synchronisation status and on-demand synchronisation per user.</t>
         </is>
       </c>
-      <c r="H9" s="12" t="inlineStr">
+      <c r="J9" s="12" t="inlineStr">
         <is>
           <t>Added by BDOI's FRS (FRUM.002.02, FRUM.003.03); not available in the system today.</t>
         </is>
       </c>
-      <c r="I9" s="12" t="inlineStr">
+      <c r="K9" s="12" t="inlineStr">
         <is>
           <t>Added by BDOI's FRS</t>
         </is>
       </c>
-      <c r="J9" s="12" t="inlineStr">
+      <c r="L9" s="12" t="inlineStr">
         <is>
           <t>Provisioning interface and user screens</t>
         </is>
       </c>
-      <c r="K9" s="12" t="inlineStr">
+      <c r="M9" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="L9" s="12" t="inlineStr">
+      <c r="N9" s="12" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="M9" s="12" t="inlineStr">
+      <c r="O9" s="12" t="inlineStr">
         <is>
           <t>All modules (users)</t>
         </is>
       </c>
-      <c r="N9" s="12" t="inlineStr">
+      <c r="P9" s="12" t="inlineStr">
         <is>
           <t>FRUM.002.02, FRUM.003.03 cases</t>
         </is>
       </c>
-      <c r="O9" s="12" t="inlineStr">
+      <c r="Q9" s="12" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="P9" s="25" t="inlineStr">
+      <c r="R9" s="25" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="Q9" s="12" t="inlineStr">
-        <is>
-          <t>Not a change request (review of 11-Oct-2026): Offered as standard (identity synchronisation with UIDM-ISC and EIAM, Synchronise Now); refines the BRD requirement 'Integration with SSO or LDAP: Yes'. No change request, no cost.</t>
-        </is>
-      </c>
-      <c r="R9" s="12" t="inlineStr">
+      <c r="S9" s="12" t="inlineStr">
+        <is>
+          <t>Not a change request (review of 11-Oct-2026): Integration scope: synchronisation of user details and status from UIDM-ISC / EIAM is an interface with BDOI's identity systems, covered by the Integration workstream (Annex AA.5). Not a change request.</t>
+        </is>
+      </c>
+      <c r="T9" s="12" t="inlineStr">
         <is>
           <t>iorta TechNXT Project Team (for BDOI confirmation)</t>
         </is>
       </c>
-      <c r="S9" s="12" t="inlineStr">
+      <c r="U9" s="12" t="inlineStr">
         <is>
           <t>11-Oct-2026</t>
         </is>
       </c>
-      <c r="T9" s="12" t="inlineStr"/>
-      <c r="U9" s="12" t="inlineStr">
+      <c r="V9" s="12" t="inlineStr"/>
+      <c r="W9" s="12" t="inlineStr">
         <is>
           <t>TC-FRUM-002.02-AC01, TC-FRUM-002.02-AC02</t>
         </is>
@@ -2624,96 +2712,106 @@
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>Offered as standard (OB-UA-05, green in the FRS)</t>
+          <t>Integration scope (IS-UA-02, grey label in the FRS)</t>
         </is>
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
+          <t>UAM-011 Directory / LDAP authentication: Not available</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
           <t>09-Oct-2026</t>
         </is>
       </c>
-      <c r="D10" s="12" t="inlineStr">
+      <c r="F10" s="12" t="inlineStr">
         <is>
           <t>iorta TechNXT Project Team</t>
         </is>
       </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="G10" s="12" t="inlineStr">
         <is>
           <t>BRD 1.004</t>
         </is>
       </c>
-      <c r="F10" s="12" t="inlineStr">
+      <c r="H10" s="12" t="inlineStr">
         <is>
           <t>FRUM.003.02.01</t>
         </is>
       </c>
-      <c r="G10" s="12" t="inlineStr">
+      <c r="I10" s="12" t="inlineStr">
         <is>
           <t>Revocation on an SSO status change: Access revoked and open sessions ended as soon as the SSO status is inactive, locked or disabled.</t>
         </is>
       </c>
-      <c r="H10" s="12" t="inlineStr">
+      <c r="J10" s="12" t="inlineStr">
         <is>
           <t>Added by BDOI's FRS (Annex Q, C13).</t>
         </is>
       </c>
-      <c r="I10" s="12" t="inlineStr">
+      <c r="K10" s="12" t="inlineStr">
         <is>
           <t>Added by BDOI's FRS</t>
         </is>
       </c>
-      <c r="J10" s="12" t="inlineStr">
+      <c r="L10" s="12" t="inlineStr">
         <is>
           <t>Status events from UIDM-ISC / EIAM</t>
         </is>
       </c>
-      <c r="K10" s="12" t="inlineStr">
+      <c r="M10" s="12" t="inlineStr">
         <is>
           <t>Small</t>
         </is>
       </c>
-      <c r="L10" s="12" t="inlineStr">
+      <c r="N10" s="12" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="M10" s="12" t="inlineStr">
+      <c r="O10" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N10" s="12" t="inlineStr">
+      <c r="P10" s="12" t="inlineStr">
         <is>
           <t>FRUM.003.02.01 cases</t>
         </is>
       </c>
-      <c r="O10" s="12" t="inlineStr">
+      <c r="Q10" s="12" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="P10" s="25" t="inlineStr">
+      <c r="R10" s="25" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="Q10" s="12" t="inlineStr">
-        <is>
-          <t>Not a change request (review of 11-Oct-2026): Offered as standard (a leaver or an inactive, locked or disabled SSO account deactivates the user and ends the sessions). No change request, no cost.</t>
-        </is>
-      </c>
-      <c r="R10" s="12" t="inlineStr">
+      <c r="S10" s="12" t="inlineStr">
+        <is>
+          <t>Not a change request (review of 11-Oct-2026): Integration scope: revocation on an SSO status change comes with the identity events of UIDM-ISC / EIAM, covered by the Integration workstream (Annex AA.5). Not a change request.</t>
+        </is>
+      </c>
+      <c r="T10" s="12" t="inlineStr">
         <is>
           <t>iorta TechNXT Project Team (for BDOI confirmation)</t>
         </is>
       </c>
-      <c r="S10" s="12" t="inlineStr">
+      <c r="U10" s="12" t="inlineStr">
         <is>
           <t>11-Oct-2026</t>
         </is>
       </c>
-      <c r="T10" s="12" t="inlineStr"/>
-      <c r="U10" s="12" t="inlineStr">
+      <c r="V10" s="12" t="inlineStr"/>
+      <c r="W10" s="12" t="inlineStr">
         <is>
           <t>TC-FRUM-003.02.01-AC01, TC-FRUM-003.02.01-AC02, TC-FRUM-003.02.01-AC03, TC-UA-006.1-01, TC-UA-006.2-01</t>
         </is>
@@ -2732,79 +2830,89 @@
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
+          <t>UAM-017 Data-scope restriction: Partial</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Partly (data scope by company and branch; no supervisor link)</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
           <t>09-Oct-2026</t>
         </is>
       </c>
-      <c r="D11" s="12" t="inlineStr">
+      <c r="F11" s="12" t="inlineStr">
         <is>
           <t>iorta TechNXT Project Team</t>
         </is>
       </c>
-      <c r="E11" s="12" t="inlineStr">
+      <c r="G11" s="12" t="inlineStr">
         <is>
           <t>Not in BRD</t>
         </is>
       </c>
-      <c r="F11" s="12" t="inlineStr">
+      <c r="H11" s="12" t="inlineStr">
         <is>
           <t>FRUM.001.02 (b), FRUM.005.01; Annex Q (C15)</t>
         </is>
       </c>
-      <c r="G11" s="12" t="inlineStr">
-        <is>
-          <t>Supervisory and record-ownership access: Supervisor (reports-to) on the user record and in the access requests; data scope "own records", "own and assigned personnel" and "unit" per group profile; the rule applied to the lists, records, documents and reports of every module; audit of the scope changes; screens of the user and the group profile.</t>
-        </is>
-      </c>
-      <c r="H11" s="12" t="inlineStr">
-        <is>
-          <t>BDOI's FRS asks that a user with a supervisory role sees and manages the records of the personnel assigned to him or her, with record-ownership rules per role. The system limits each user's data by company and branch (data scope) and by role; it has no supervisor-to-personnel link and no record-owner rule.</t>
-        </is>
-      </c>
       <c r="I11" s="12" t="inlineStr">
         <is>
+          <t>Supervisory and record-ownership access: Data scope by company, branch and unit on the user and the group profile; supervisor (reports-to) on the user record and in the access requests; data scope "own records", "own and assigned personnel" and "unit" per group profile; the rule applied to the lists, records, documents and reports of every module; audit of the scope changes; screens of the user and the group profile.</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="inlineStr">
+        <is>
+          <t>BDOI's FRS asks that a user with a supervisory role sees and manages the records of the personnel assigned to him or her, with record-ownership rules per role. The OOTB platform limits scoped roles to their own records and clients (UAM-017 Partial); it has no scope by branch or unit, no supervisor-to-personnel link and no record-owner rule per role.</t>
+        </is>
+      </c>
+      <c r="K11" s="12" t="inlineStr">
+        <is>
           <t>Added by BDOI's FRS</t>
         </is>
       </c>
-      <c r="J11" s="12" t="inlineStr">
+      <c r="L11" s="12" t="inlineStr">
         <is>
           <t>Rules per role</t>
         </is>
       </c>
-      <c r="K11" s="12" t="inlineStr">
+      <c r="M11" s="12" t="inlineStr">
         <is>
           <t>High complexity</t>
         </is>
       </c>
-      <c r="L11" s="12" t="inlineStr">
-        <is>
-          <t>23 man-days (CR Effort Estimate)</t>
-        </is>
-      </c>
-      <c r="M11" s="12" t="inlineStr">
+      <c r="N11" s="12" t="inlineStr">
+        <is>
+          <t>27.5 man-days (CR Effort Estimate)</t>
+        </is>
+      </c>
+      <c r="O11" s="12" t="inlineStr">
         <is>
           <t>All modules (data scope)</t>
         </is>
       </c>
-      <c r="N11" s="12" t="inlineStr">
+      <c r="P11" s="12" t="inlineStr">
         <is>
           <t>FRUM.005.01 cases</t>
         </is>
       </c>
-      <c r="O11" s="12" t="inlineStr">
+      <c r="Q11" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="P11" s="25" t="inlineStr">
+      <c r="R11" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q11" s="12" t="inlineStr"/>
-      <c r="R11" s="12" t="inlineStr"/>
       <c r="S11" s="12" t="inlineStr"/>
       <c r="T11" s="12" t="inlineStr"/>
-      <c r="U11" s="12" t="inlineStr">
+      <c r="U11" s="12" t="inlineStr"/>
+      <c r="V11" s="12" t="inlineStr"/>
+      <c r="W11" s="12" t="inlineStr">
         <is>
           <t>TC-FRUM-005.01-AC01, TC-FRUM-005.01-AC02, TC-FRUM-005.01-AC03, TC-UA-040.1-01, TC-UA-040.2-01</t>
         </is>
@@ -2818,96 +2926,94 @@
       </c>
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>Offered as standard (OB-UA-06, green in the FRS)</t>
+          <t>Change request (orange in the FRS)</t>
         </is>
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
+          <t>UAM-018 Segregation of duties rules: Available (pairs of roles only)</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
           <t>09-Oct-2026</t>
         </is>
       </c>
-      <c r="D12" s="12" t="inlineStr">
+      <c r="F12" s="12" t="inlineStr">
         <is>
           <t>iorta TechNXT Project Team</t>
         </is>
       </c>
-      <c r="E12" s="12" t="inlineStr">
-        <is>
-          <t>BRD 4.002.2</t>
-        </is>
-      </c>
-      <c r="F12" s="12" t="inlineStr">
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>Not in BRD</t>
+        </is>
+      </c>
+      <c r="H12" s="12" t="inlineStr">
         <is>
           <t>FRUM.006.03</t>
         </is>
       </c>
-      <c r="G12" s="12" t="inlineStr">
-        <is>
-          <t>Conflicting permission combinations inside a role: A role cannot hold two permissions that conflict.</t>
-        </is>
-      </c>
-      <c r="H12" s="12" t="inlineStr">
-        <is>
-          <t>Added by BDOI's FRS (Annex Q, C16); the system checks pairs of profiles today.</t>
-        </is>
-      </c>
       <c r="I12" s="12" t="inlineStr">
         <is>
+          <t>No conflicting permissions inside a group profile: Rules on pairs of permissions kept by the Business Administrator; check on every group profile change and access request; message naming the conflict; audit.</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="inlineStr">
+        <is>
+          <t>BDOI's FRS asks that a group profile cannot hold two permissions that conflict. The OOTB platform checks pairs of roles held by one user (separation-of-duties rules); it has no rule on pairs of permissions inside a role.</t>
+        </is>
+      </c>
+      <c r="K12" s="12" t="inlineStr">
+        <is>
           <t>Added by BDOI's FRS</t>
         </is>
       </c>
-      <c r="J12" s="12" t="inlineStr">
+      <c r="L12" s="12" t="inlineStr">
         <is>
           <t>Rule on permission pairs</t>
         </is>
       </c>
-      <c r="K12" s="12" t="inlineStr">
-        <is>
-          <t>Small</t>
-        </is>
-      </c>
-      <c r="L12" s="12" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="M12" s="12" t="inlineStr">
         <is>
+          <t>Low complexity</t>
+        </is>
+      </c>
+      <c r="N12" s="12" t="inlineStr">
+        <is>
+          <t>4.75 man-days (CR Effort Estimate)</t>
+        </is>
+      </c>
+      <c r="O12" s="12" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N12" s="12" t="inlineStr">
+      <c r="P12" s="12" t="inlineStr">
         <is>
           <t>FRUM.006.03 cases</t>
         </is>
       </c>
-      <c r="O12" s="12" t="inlineStr">
+      <c r="Q12" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="P12" s="25" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="Q12" s="12" t="inlineStr">
-        <is>
-          <t>Not a change request (review of 11-Oct-2026): Offered as standard (rules on permission pairs, checked on roles and on users). No change request, no cost.</t>
-        </is>
-      </c>
-      <c r="R12" s="12" t="inlineStr">
-        <is>
-          <t>iorta TechNXT Project Team (for BDOI confirmation)</t>
-        </is>
-      </c>
-      <c r="S12" s="12" t="inlineStr">
-        <is>
-          <t>11-Oct-2026</t>
-        </is>
-      </c>
+      <c r="R12" s="25" t="inlineStr">
+        <is>
+          <t>Candidate - for decision</t>
+        </is>
+      </c>
+      <c r="S12" s="12" t="inlineStr"/>
       <c r="T12" s="12" t="inlineStr"/>
-      <c r="U12" s="12" t="inlineStr">
+      <c r="U12" s="12" t="inlineStr"/>
+      <c r="V12" s="12" t="inlineStr"/>
+      <c r="W12" s="12" t="inlineStr">
         <is>
           <t>TC-FRUM-006.03-AC01, TC-FRUM-006.03-AC02, TC-UA-041.1-01, TC-UA-041.2-01, TC-UA-041.2-02</t>
         </is>
@@ -2921,96 +3027,94 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>Offered as standard (OB-UA-07, green in the FRS)</t>
+          <t>Change request (orange in the FRS)</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
+          <t>RPT-009 Report file naming conventions: Not available</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
           <t>09-Oct-2026</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="F13" s="12" t="inlineStr">
         <is>
           <t>iorta TechNXT Project Team</t>
         </is>
       </c>
-      <c r="E13" s="12" t="inlineStr">
-        <is>
-          <t>BRD p.18</t>
-        </is>
-      </c>
-      <c r="F13" s="12" t="inlineStr">
-        <is>
-          <t>FRUM.007.02</t>
-        </is>
-      </c>
       <c r="G13" s="12" t="inlineStr">
         <is>
-          <t>Export file names: Exports named &lt;Report_Name&gt;_MMDDYYYY and Audit Logs_MMDDYYYY.</t>
+          <t>Not in BRD</t>
         </is>
       </c>
       <c r="H13" s="12" t="inlineStr">
         <is>
-          <t>Added by BDOI's FRS (Annex Q, C18).</t>
+          <t>FRUM.007.02; Annex V</t>
         </is>
       </c>
       <c r="I13" s="12" t="inlineStr">
         <is>
+          <t>Export file names: File names of the User Access reports and of the audit log export by BDOI's convention, as a setting; test of every export.</t>
+        </is>
+      </c>
+      <c r="J13" s="12" t="inlineStr">
+        <is>
+          <t>BDOI's FRS names the exports &lt;Report name&gt;_MMDDYYYY and Audit Logs_MMDDYYYY. In the OOTB platform the file names are fixed per report (RPT-009 Not available).</t>
+        </is>
+      </c>
+      <c r="K13" s="12" t="inlineStr">
+        <is>
           <t>Added by BDOI's FRS</t>
         </is>
       </c>
-      <c r="J13" s="12" t="inlineStr">
+      <c r="L13" s="12" t="inlineStr">
         <is>
           <t>File name of the downloads</t>
         </is>
       </c>
-      <c r="K13" s="12" t="inlineStr">
-        <is>
-          <t>Small</t>
-        </is>
-      </c>
-      <c r="L13" s="12" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="M13" s="12" t="inlineStr">
         <is>
+          <t>Low complexity</t>
+        </is>
+      </c>
+      <c r="N13" s="12" t="inlineStr">
+        <is>
+          <t>2.25 man-days (CR Effort Estimate)</t>
+        </is>
+      </c>
+      <c r="O13" s="12" t="inlineStr">
+        <is>
           <t>All reports (common)</t>
         </is>
       </c>
-      <c r="N13" s="12" t="inlineStr">
+      <c r="P13" s="12" t="inlineStr">
         <is>
           <t>FRUM.007.02 cases</t>
         </is>
       </c>
-      <c r="O13" s="12" t="inlineStr">
+      <c r="Q13" s="12" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="P13" s="25" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="Q13" s="12" t="inlineStr">
-        <is>
-          <t>Not a change request (review of 11-Oct-2026): Offered as standard (exports named &lt;Report name&gt;_MMDDYYYY and Audit Logs_MMDDYYYY). No change request, no cost.</t>
-        </is>
-      </c>
-      <c r="R13" s="12" t="inlineStr">
-        <is>
-          <t>iorta TechNXT Project Team (for BDOI confirmation)</t>
-        </is>
-      </c>
-      <c r="S13" s="12" t="inlineStr">
-        <is>
-          <t>11-Oct-2026</t>
-        </is>
-      </c>
+      <c r="R13" s="25" t="inlineStr">
+        <is>
+          <t>Candidate - for decision</t>
+        </is>
+      </c>
+      <c r="S13" s="12" t="inlineStr"/>
       <c r="T13" s="12" t="inlineStr"/>
-      <c r="U13" s="12" t="inlineStr">
+      <c r="U13" s="12" t="inlineStr"/>
+      <c r="V13" s="12" t="inlineStr"/>
+      <c r="W13" s="12" t="inlineStr">
         <is>
           <t>TC-FRUM-007.02-AC01, TC-UA-060.1-01, TC-UA-060.1-02, TC-UA-060.2-01, TC-UA-060.3-01</t>
         </is>
@@ -3029,91 +3133,101 @@
       </c>
       <c r="C14" s="12" t="inlineStr">
         <is>
+          <t>UAM-031 Access-change log: Available</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
           <t>09-Oct-2026</t>
         </is>
       </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="F14" s="12" t="inlineStr">
         <is>
           <t>iorta TechNXT Project Team</t>
         </is>
       </c>
-      <c r="E14" s="12" t="inlineStr">
+      <c r="G14" s="12" t="inlineStr">
         <is>
           <t>NFR 4.03 of the Claims, Collections and ReInsurance addenda</t>
         </is>
       </c>
-      <c r="F14" s="12" t="inlineStr">
+      <c r="H14" s="12" t="inlineStr">
         <is>
           <t>FRUM.008.01</t>
         </is>
       </c>
-      <c r="G14" s="12" t="inlineStr">
+      <c r="I14" s="12" t="inlineStr">
         <is>
           <t>IP address and role in the audit log: Each audit record shows the source IP address and the role of the user at the time.</t>
         </is>
       </c>
-      <c r="H14" s="12" t="inlineStr">
+      <c r="J14" s="12" t="inlineStr">
         <is>
           <t>Added by BDOI's FRS (Annex Q, C19).</t>
         </is>
       </c>
-      <c r="I14" s="12" t="inlineStr">
+      <c r="K14" s="12" t="inlineStr">
         <is>
           <t>Added by BDOI's FRS</t>
         </is>
       </c>
-      <c r="J14" s="12" t="inlineStr">
+      <c r="L14" s="12" t="inlineStr">
         <is>
           <t>Audit record and report</t>
         </is>
       </c>
-      <c r="K14" s="12" t="inlineStr">
+      <c r="M14" s="12" t="inlineStr">
         <is>
           <t>Small</t>
         </is>
       </c>
-      <c r="L14" s="12" t="inlineStr">
+      <c r="N14" s="12" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="M14" s="12" t="inlineStr">
+      <c r="O14" s="12" t="inlineStr">
         <is>
           <t>All modules (audit)</t>
         </is>
       </c>
-      <c r="N14" s="12" t="inlineStr">
+      <c r="P14" s="12" t="inlineStr">
         <is>
           <t>FRUM.008 cases</t>
         </is>
       </c>
-      <c r="O14" s="12" t="inlineStr">
+      <c r="Q14" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="P14" s="25" t="inlineStr">
+      <c r="R14" s="25" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="Q14" s="12" t="inlineStr">
-        <is>
-          <t>Not a change request (review of 11-Oct-2026): Already a BRD requirement: NFR 4.03 of the Claims, Collections and ReInsurance addenda (source workstation, device or IP address of each audit event). Offered as standard.</t>
-        </is>
-      </c>
-      <c r="R14" s="12" t="inlineStr">
+      <c r="S14" s="12" t="inlineStr">
+        <is>
+          <t>Not a change request (review of 11-Oct-2026): Already a BRD requirement: NFR 4.03 of the Claims, Collections and ReInsurance addenda (source workstation, device or IP address of each audit event). Met by the OOTB platform.</t>
+        </is>
+      </c>
+      <c r="T14" s="12" t="inlineStr">
         <is>
           <t>iorta TechNXT Project Team (for BDOI confirmation)</t>
         </is>
       </c>
-      <c r="S14" s="12" t="inlineStr">
+      <c r="U14" s="12" t="inlineStr">
         <is>
           <t>11-Oct-2026</t>
         </is>
       </c>
-      <c r="T14" s="12" t="inlineStr"/>
-      <c r="U14" s="12" t="inlineStr">
+      <c r="V14" s="12" t="inlineStr"/>
+      <c r="W14" s="12" t="inlineStr">
         <is>
           <t>TC-FRUM-008.01-AC01, TC-FRUM-008.01-AC02, TC-UA-004.1-01, TC-UA-004.2-01, TC-UA-004.3-01</t>
         </is>
@@ -3132,79 +3246,89 @@
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
+          <t>WFL-007 Turnaround-time tracking and escalation: Partial (UAM-019 access requests: Not available)</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
           <t>09-Oct-2026</t>
         </is>
       </c>
-      <c r="D15" s="12" t="inlineStr">
+      <c r="F15" s="12" t="inlineStr">
         <is>
           <t>iorta TechNXT Project Team</t>
         </is>
       </c>
-      <c r="E15" s="12" t="inlineStr">
+      <c r="G15" s="12" t="inlineStr">
         <is>
           <t>Not in BRD</t>
         </is>
       </c>
-      <c r="F15" s="12" t="inlineStr">
+      <c r="H15" s="12" t="inlineStr">
         <is>
           <t>Annex S (time rules), Annex Q.5, Annex Z</t>
         </is>
       </c>
-      <c r="G15" s="12" t="inlineStr">
+      <c r="I15" s="12" t="inlineStr">
         <is>
           <t>Approval times, reminders and escalation: Settings for the working days per stage, the reminder day and the escalation role; a daily run that sends the reminder notice and escalates overdue requests to the Business Administrator; the overdue marker on the lists; audit of each reminder and escalation.</t>
         </is>
       </c>
-      <c r="H15" s="12" t="inlineStr">
-        <is>
-          <t>The BRD sets no service level for the approval of access requests. Today the age of each request shows on the Access Requests list and report; a reminder and an escalation after a number of working days keep requests from waiting unseen.</t>
-        </is>
-      </c>
-      <c r="I15" s="12" t="inlineStr">
+      <c r="J15" s="12" t="inlineStr">
+        <is>
+          <t>The BRD sets no service level for the approval of access requests. A reminder and an escalation after a number of working days keep requests from waiting unseen. The OOTB platform has deadlines and escalation for claims, complaints, leads and collections only, and no access requests (WFL-007 Partial).</t>
+        </is>
+      </c>
+      <c r="K15" s="12" t="inlineStr">
         <is>
           <t>Beyond the BRD</t>
         </is>
       </c>
-      <c r="J15" s="12" t="inlineStr">
+      <c r="L15" s="12" t="inlineStr">
         <is>
           <t>Reminder and escalation run</t>
         </is>
       </c>
-      <c r="K15" s="12" t="inlineStr">
+      <c r="M15" s="12" t="inlineStr">
         <is>
           <t>Medium complexity</t>
         </is>
       </c>
-      <c r="L15" s="12" t="inlineStr">
+      <c r="N15" s="12" t="inlineStr">
         <is>
           <t>8 man-days (CR Effort Estimate)</t>
         </is>
       </c>
-      <c r="M15" s="12" t="inlineStr">
+      <c r="O15" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N15" s="12" t="inlineStr">
+      <c r="P15" s="12" t="inlineStr">
         <is>
           <t>FRUM.010 cases</t>
         </is>
       </c>
-      <c r="O15" s="12" t="inlineStr">
+      <c r="Q15" s="12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="P15" s="25" t="inlineStr">
+      <c r="R15" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q15" s="12" t="inlineStr"/>
-      <c r="R15" s="12" t="inlineStr"/>
       <c r="S15" s="12" t="inlineStr"/>
       <c r="T15" s="12" t="inlineStr"/>
-      <c r="U15" s="12" t="inlineStr">
+      <c r="U15" s="12" t="inlineStr"/>
+      <c r="V15" s="12" t="inlineStr"/>
+      <c r="W15" s="12" t="inlineStr">
         <is>
           <t>TC-FRUM-010.01-AC01, TC-FRUM-010.01-AC02, TC-UA-030.1-01, TC-UA-030.2-01, TC-UA-030.3-01</t>
         </is>
@@ -3218,84 +3342,106 @@
       </c>
       <c r="B16" s="12" t="inlineStr">
         <is>
-          <t>Change request (orange in the FRS)</t>
+          <t>Offered by iNXT BrokerVerse OOTB (OB-UA-05, green in the FRS)</t>
         </is>
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
+          <t>UAM-030 Periodic access entitlement review: Available; RPT-007 User-scheduled reports: Available</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
           <t>09-Oct-2026</t>
         </is>
       </c>
-      <c r="D16" s="12" t="inlineStr">
+      <c r="F16" s="12" t="inlineStr">
         <is>
           <t>iorta TechNXT Project Team</t>
         </is>
       </c>
-      <c r="E16" s="12" t="inlineStr">
-        <is>
-          <t>Not in BRD (BRD p.11 lists report volumes only)</t>
-        </is>
-      </c>
-      <c r="F16" s="12" t="inlineStr">
-        <is>
-          <t>Annex V, Annex Q.5 (UA-Q51)</t>
-        </is>
-      </c>
       <c r="G16" s="12" t="inlineStr">
         <is>
-          <t>Monthly access review report to Information Security: A monthly run on the first working day that produces the User Access Report and the audit log of the month, keeps the files for download and notifies Information Security (in the system and by e-mail, with no attachment); run history and failure notice as for the other runs.</t>
+          <t>BRD NFR p.11</t>
         </is>
       </c>
       <c r="H16" s="12" t="inlineStr">
         <is>
-          <t>Information Security practice is a periodic review of who holds which access. The reports exist and run on demand; producing them each month for Information Security makes the review routine.</t>
+          <t>FRUM.007</t>
         </is>
       </c>
       <c r="I16" s="12" t="inlineStr">
         <is>
-          <t>Beyond the BRD</t>
+          <t>Monthly access review report: User Access Report and audit log of the month sent to Information Security on the first working day.</t>
         </is>
       </c>
       <c r="J16" s="12" t="inlineStr">
         <is>
+          <t>Best practice; UA-Q51 (Annex Q.5).</t>
+        </is>
+      </c>
+      <c r="K16" s="12" t="inlineStr">
+        <is>
+          <t>Proposal for best practice</t>
+        </is>
+      </c>
+      <c r="L16" s="12" t="inlineStr">
+        <is>
           <t>Scheduled report</t>
         </is>
       </c>
-      <c r="K16" s="12" t="inlineStr">
-        <is>
-          <t>Low complexity</t>
-        </is>
-      </c>
-      <c r="L16" s="12" t="inlineStr">
-        <is>
-          <t>6 man-days (CR Effort Estimate)</t>
-        </is>
-      </c>
       <c r="M16" s="12" t="inlineStr">
         <is>
+          <t>Small</t>
+        </is>
+      </c>
+      <c r="N16" s="12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="O16" s="12" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N16" s="12" t="inlineStr">
+      <c r="P16" s="12" t="inlineStr">
         <is>
           <t>FRUM.007 cases</t>
         </is>
       </c>
-      <c r="O16" s="12" t="inlineStr">
+      <c r="Q16" s="12" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="P16" s="25" t="inlineStr">
-        <is>
-          <t>Candidate - for decision</t>
-        </is>
-      </c>
-      <c r="Q16" s="12" t="inlineStr"/>
-      <c r="R16" s="12" t="inlineStr"/>
-      <c r="S16" s="12" t="inlineStr"/>
-      <c r="T16" s="12" t="inlineStr"/>
+      <c r="R16" s="25" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="S16" s="12" t="inlineStr">
+        <is>
+          <t>Not a change request (review of 11-Oct-2026): Offered by the iNXT BrokerVerse OOTB platform (periodic access entitlement review; report schedules with recipients). No change request, no cost; the BDOI report layouts are BRD work (BRD-UA-15).</t>
+        </is>
+      </c>
+      <c r="T16" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team (for BDOI confirmation)</t>
+        </is>
+      </c>
       <c r="U16" s="12" t="inlineStr">
+        <is>
+          <t>11-Oct-2026</t>
+        </is>
+      </c>
+      <c r="V16" s="12" t="inlineStr"/>
+      <c r="W16" s="12" t="inlineStr">
         <is>
           <t>TC-FRUM-007.01-AC01, TC-FRUM-007.01-AC02, TC-FRUM-007.01-AC03, TC-UA-060.1-01, TC-UA-060.1-02</t>
         </is>
@@ -3309,96 +3455,94 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>Offered as standard (OB-UA-08, green in the FRS)</t>
+          <t>Change request (orange in the FRS)</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
+          <t>UAM-027 Notices of access changes: Partial</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
           <t>09-Oct-2026</t>
         </is>
       </c>
-      <c r="D17" s="12" t="inlineStr">
+      <c r="F17" s="12" t="inlineStr">
         <is>
           <t>iorta TechNXT Project Team</t>
         </is>
       </c>
-      <c r="E17" s="12" t="inlineStr">
-        <is>
-          <t>BRD 1.006.1.1, 1.008.1.4, 2.002.1</t>
-        </is>
-      </c>
-      <c r="F17" s="12" t="inlineStr">
-        <is>
-          <t>FRUM.013.01</t>
-        </is>
-      </c>
       <c r="G17" s="12" t="inlineStr">
         <is>
-          <t>E-mail copy of the request notices: The notices to approve, returned and decided also sent by e-mail by the user's preference.</t>
+          <t>Not in BRD</t>
         </is>
       </c>
       <c r="H17" s="12" t="inlineStr">
         <is>
-          <t>The BRD asks for a notification (met in the system); Annex Z.</t>
+          <t>FRUM.013.01; Annex T</t>
         </is>
       </c>
       <c r="I17" s="12" t="inlineStr">
         <is>
-          <t>Proposal for best practice</t>
+          <t>E-mail copy of the request notices: E-mail copy of the request notices (to approve, returned, decided) from templates, by the user's preference (setting); the outbox status; tests.</t>
         </is>
       </c>
       <c r="J17" s="12" t="inlineStr">
         <is>
+          <t>BDOI's FRS asks that the notices to approve, returned and decided are also e-mailed, by the user's preference. The OOTB platform sends in-system notices for access-control events (UAM-027 Partial); it has e-mail templates (WFL-011) but no e-mail copy of the access notices.</t>
+        </is>
+      </c>
+      <c r="K17" s="12" t="inlineStr">
+        <is>
+          <t>Beyond the BRD</t>
+        </is>
+      </c>
+      <c r="L17" s="12" t="inlineStr">
+        <is>
           <t>E-mail of the notices</t>
         </is>
       </c>
-      <c r="K17" s="12" t="inlineStr">
-        <is>
-          <t>Small</t>
-        </is>
-      </c>
-      <c r="L17" s="12" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="M17" s="12" t="inlineStr">
         <is>
+          <t>Low complexity</t>
+        </is>
+      </c>
+      <c r="N17" s="12" t="inlineStr">
+        <is>
+          <t>3.75 man-days (CR Effort Estimate)</t>
+        </is>
+      </c>
+      <c r="O17" s="12" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N17" s="12" t="inlineStr">
+      <c r="P17" s="12" t="inlineStr">
         <is>
           <t>FRUM.013.01 cases</t>
         </is>
       </c>
-      <c r="O17" s="12" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="P17" s="25" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
       <c r="Q17" s="12" t="inlineStr">
         <is>
-          <t>Not a change request (review of 11-Oct-2026): Offered as standard (setting: request notices also e-mailed by the user's preference). No change request, no cost.</t>
-        </is>
-      </c>
-      <c r="R17" s="12" t="inlineStr">
-        <is>
-          <t>iorta TechNXT Project Team (for BDOI confirmation)</t>
-        </is>
-      </c>
-      <c r="S17" s="12" t="inlineStr">
-        <is>
-          <t>11-Oct-2026</t>
-        </is>
-      </c>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R17" s="25" t="inlineStr">
+        <is>
+          <t>Candidate - for decision</t>
+        </is>
+      </c>
+      <c r="S17" s="12" t="inlineStr"/>
       <c r="T17" s="12" t="inlineStr"/>
-      <c r="U17" s="12" t="inlineStr">
+      <c r="U17" s="12" t="inlineStr"/>
+      <c r="V17" s="12" t="inlineStr"/>
+      <c r="W17" s="12" t="inlineStr">
         <is>
           <t>TC-FRUM-013.01-AC01, TC-FRUM-013.01-AC02, TC-UA-070.1-01, TC-UA-070.2-01, TC-UA-070.3-01</t>
         </is>
@@ -3417,79 +3561,89 @@
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
+          <t>UAM-024 Effective-dated access changes: Not available</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
           <t>09-Oct-2026</t>
         </is>
       </c>
-      <c r="D18" s="12" t="inlineStr">
+      <c r="F18" s="12" t="inlineStr">
         <is>
           <t>iorta TechNXT Project Team</t>
         </is>
       </c>
-      <c r="E18" s="12" t="inlineStr">
+      <c r="G18" s="12" t="inlineStr">
         <is>
           <t>Not in BRD (BRD NFR 1.k asks for an effective date only)</t>
         </is>
       </c>
-      <c r="F18" s="12" t="inlineStr">
+      <c r="H18" s="12" t="inlineStr">
         <is>
           <t>Annex Z (CLR-UA-06, CLR-UA-13); FRUM.009.10</t>
         </is>
       </c>
-      <c r="G18" s="12" t="inlineStr">
+      <c r="I18" s="12" t="inlineStr">
         <is>
           <t>Temporary access with an end date: End date on the user requests and the bulk template; validation (after the effective date); the end date on the user's group profiles and in the reports; the daily run removes the access on the end date with a notice a number of days before; audit of each removal.</t>
         </is>
       </c>
-      <c r="H18" s="12" t="inlineStr">
-        <is>
-          <t>Access given for a project or a leave cover should end by itself. The system applies changes on an effective date; it has no end date on access.</t>
-        </is>
-      </c>
-      <c r="I18" s="12" t="inlineStr">
+      <c r="J18" s="12" t="inlineStr">
+        <is>
+          <t>Access given for a project or a leave cover should end by itself. The OOTB platform applies changes at once, with no effective or end date (UAM-024 Not available); the effective date is a BRD requirement (Annex AA.4).</t>
+        </is>
+      </c>
+      <c r="K18" s="12" t="inlineStr">
         <is>
           <t>Beyond the BRD</t>
         </is>
       </c>
-      <c r="J18" s="12" t="inlineStr">
+      <c r="L18" s="12" t="inlineStr">
         <is>
           <t>End date on requests</t>
         </is>
       </c>
-      <c r="K18" s="12" t="inlineStr">
+      <c r="M18" s="12" t="inlineStr">
         <is>
           <t>Medium complexity</t>
         </is>
       </c>
-      <c r="L18" s="12" t="inlineStr">
+      <c r="N18" s="12" t="inlineStr">
         <is>
           <t>11.5 man-days (CR Effort Estimate)</t>
         </is>
       </c>
-      <c r="M18" s="12" t="inlineStr">
+      <c r="O18" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="N18" s="12" t="inlineStr">
+      <c r="P18" s="12" t="inlineStr">
         <is>
           <t>FRUM.009.10 cases</t>
         </is>
       </c>
-      <c r="O18" s="12" t="inlineStr">
+      <c r="Q18" s="12" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="P18" s="25" t="inlineStr">
+      <c r="R18" s="25" t="inlineStr">
         <is>
           <t>Candidate - for decision</t>
         </is>
       </c>
-      <c r="Q18" s="12" t="inlineStr"/>
-      <c r="R18" s="12" t="inlineStr"/>
       <c r="S18" s="12" t="inlineStr"/>
       <c r="T18" s="12" t="inlineStr"/>
-      <c r="U18" s="12" t="inlineStr">
+      <c r="U18" s="12" t="inlineStr"/>
+      <c r="V18" s="12" t="inlineStr"/>
+      <c r="W18" s="12" t="inlineStr">
         <is>
           <t>TC-FRUM-009.10-AC01, TC-FRUM-009.10-AC02, TC-UA-020.1-01, TC-UA-020.2-01, TC-UA-020.3-01</t>
         </is>
@@ -3508,119 +3662,230 @@
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
+          <t>UAM-005 Single session per user or device: Not available</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
           <t>09-Oct-2026</t>
         </is>
       </c>
-      <c r="D19" s="12" t="inlineStr">
+      <c r="F19" s="12" t="inlineStr">
         <is>
           <t>iorta TechNXT Project Team</t>
         </is>
       </c>
-      <c r="E19" s="12" t="inlineStr">
+      <c r="G19" s="12" t="inlineStr">
         <is>
           <t>NFR 10.07 of the Collections addendum</t>
         </is>
       </c>
-      <c r="F19" s="12" t="inlineStr">
+      <c r="H19" s="12" t="inlineStr">
         <is>
           <t>FRUM.001.01</t>
         </is>
       </c>
-      <c r="G19" s="12" t="inlineStr">
+      <c r="I19" s="12" t="inlineStr">
         <is>
           <t>One session per user or device: A new sign-in ends the earlier session of the same user (or device).</t>
         </is>
       </c>
-      <c r="H19" s="12" t="inlineStr">
+      <c r="J19" s="12" t="inlineStr">
         <is>
           <t>Open question CLR-UA-09 (Annex Z).</t>
         </is>
       </c>
-      <c r="I19" s="12" t="inlineStr">
+      <c r="K19" s="12" t="inlineStr">
         <is>
           <t>Beyond the BRD</t>
         </is>
       </c>
-      <c r="J19" s="12" t="inlineStr">
+      <c r="L19" s="12" t="inlineStr">
         <is>
           <t>Session rule</t>
         </is>
       </c>
-      <c r="K19" s="12" t="inlineStr">
+      <c r="M19" s="12" t="inlineStr">
         <is>
           <t>Small</t>
         </is>
       </c>
-      <c r="L19" s="12" t="inlineStr">
+      <c r="N19" s="12" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="M19" s="12" t="inlineStr">
+      <c r="O19" s="12" t="inlineStr">
         <is>
           <t>All users</t>
         </is>
       </c>
-      <c r="N19" s="12" t="inlineStr">
+      <c r="P19" s="12" t="inlineStr">
         <is>
           <t>FRUM.001 cases</t>
         </is>
       </c>
-      <c r="O19" s="12" t="inlineStr">
+      <c r="Q19" s="12" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="P19" s="25" t="inlineStr">
+      <c r="R19" s="25" t="inlineStr">
         <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="Q19" s="12" t="inlineStr">
-        <is>
-          <t>Not a change request (review of 11-Oct-2026): Already a BRD requirement: NFR 10.07 of the Collections addendum (one session per device; a sign-in on another device ends the earlier session). In scope; to be delivered before UAT (Annex AA.4).</t>
-        </is>
-      </c>
-      <c r="R19" s="12" t="inlineStr">
+      <c r="S19" s="12" t="inlineStr">
+        <is>
+          <t>Not a change request (review of 11-Oct-2026): Already a BRD requirement: NFR 10.07 of the Collections addendum (one session per device; a sign-in on another device ends the earlier session). Not in the OOTB platform; in scope, to be delivered before UAT (BRD-UA-01, Annex AA.4).</t>
+        </is>
+      </c>
+      <c r="T19" s="12" t="inlineStr">
         <is>
           <t>iorta TechNXT Project Team (for BDOI confirmation)</t>
         </is>
       </c>
-      <c r="S19" s="12" t="inlineStr">
+      <c r="U19" s="12" t="inlineStr">
         <is>
           <t>11-Oct-2026</t>
         </is>
       </c>
-      <c r="T19" s="12" t="inlineStr"/>
-      <c r="U19" s="12" t="inlineStr">
+      <c r="V19" s="12" t="inlineStr"/>
+      <c r="W19" s="12" t="inlineStr">
         <is>
           <t>TC-FRUM-001.01-AC01, TC-FRUM-001.01-AC02, TC-UA-001.1-01, TC-UA-001.1-02, TC-UA-001.2-01</t>
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>CR-UA-016</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>Change request (orange in the FRS)</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>No feature row (UAM-022 group profile requests: Not available)</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>09-Oct-2026</t>
+        </is>
+      </c>
+      <c r="F20" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="G20" s="12" t="inlineStr">
+        <is>
+          <t>Not in BRD</t>
+        </is>
+      </c>
+      <c r="H20" s="12" t="inlineStr">
+        <is>
+          <t>FRUM.005.01; Annex J</t>
+        </is>
+      </c>
+      <c r="I20" s="12" t="inlineStr">
+        <is>
+          <t>Emergency role edit: The emergency role edit setting, opened by Information Security; the direct edit of users and group profiles by the System Administrator while it is open, closed as delivered; every edit audited and alerted to Information Security; the marker on the screens.</t>
+        </is>
+      </c>
+      <c r="J20" s="12" t="inlineStr">
+        <is>
+          <t>With group profiles changed only by approved requests, an emergency path lets the System Administrator edit users and group profiles directly, when Information Security opens it, with every edit audited and alerted. The OOTB platform has no request flow and no emergency edit; the feature list has no row for it.</t>
+        </is>
+      </c>
+      <c r="K20" s="12" t="inlineStr">
+        <is>
+          <t>Beyond the BRD</t>
+        </is>
+      </c>
+      <c r="L20" s="12" t="inlineStr">
+        <is>
+          <t>Emergency edit setting, audit and alert</t>
+        </is>
+      </c>
+      <c r="M20" s="12" t="inlineStr">
+        <is>
+          <t>Medium complexity</t>
+        </is>
+      </c>
+      <c r="N20" s="12" t="inlineStr">
+        <is>
+          <t>6.5 man-days (CR Effort Estimate)</t>
+        </is>
+      </c>
+      <c r="O20" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P20" s="12" t="inlineStr">
+        <is>
+          <t>FRUM.005.01 cases</t>
+        </is>
+      </c>
+      <c r="Q20" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R20" s="25" t="inlineStr">
+        <is>
+          <t>Candidate - for decision</t>
+        </is>
+      </c>
+      <c r="S20" s="12" t="inlineStr"/>
+      <c r="T20" s="12" t="inlineStr"/>
+      <c r="U20" s="12" t="inlineStr"/>
+      <c r="V20" s="12" t="inlineStr"/>
+      <c r="W20" s="12" t="inlineStr">
+        <is>
+          <t>TC-FRUM-005.01-AC01, TC-FRUM-005.01-AC02, TC-FRUM-005.01-AC03, TC-UA-040.1-01, TC-UA-040.2-01</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:U19"/>
+  <autoFilter ref="A4:W20"/>
   <mergeCells count="1">
-    <mergeCell ref="A2:U2"/>
+    <mergeCell ref="A2:W2"/>
   </mergeCells>
-  <conditionalFormatting sqref="P5:P519">
+  <conditionalFormatting sqref="R5:R520">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="1" stopIfTrue="1">
       <formula>"Closed"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:U519">
+  <conditionalFormatting sqref="A5:W520">
     <cfRule type="expression" priority="2" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="I5:I519" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
+    <dataValidation sqref="K5:K520" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
       <formula1>'Lists'!$A$2:$A$5</formula1>
     </dataValidation>
-    <dataValidation sqref="O5:O519" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Priority" error="Choose a value from the list (Priority)." type="list">
+    <dataValidation sqref="Q5:Q520" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Priority" error="Choose a value from the list (Priority)." type="list">
       <formula1>'Lists'!$B$2:$B$4</formula1>
     </dataValidation>
-    <dataValidation sqref="P5:P519" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
+    <dataValidation sqref="R5:R520" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
       <formula1>'Lists'!$C$2:$C$9</formula1>
     </dataValidation>
   </dataValidations>
@@ -6661,7 +6926,7 @@
       </c>
       <c r="D77" s="12" t="inlineStr">
         <is>
-          <t>Proposed as best practice: the User Access Report and the User Access Audit Log of the month sent to Information Security on the first working day of each month. Not available today (reports run on demand).</t>
+          <t>Proposed as best practice: the User Access Report and the User Access Audit Log of the month sent to Information Security on the first working day of each month, with the report schedules and periodic access reviews of the iNXT BrokerVerse OOTB platform.</t>
         </is>
       </c>
       <c r="E77" s="12" t="inlineStr">

</xml_diff>

<commit_message>
UAM FRS v1.4: column Prepared for BIBS?, minimum column width in the shared table refit, rebuilt after merging Renewal v1.2
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W3DAuLtsQmip7EuxjJCCtN
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-11_User_Access_Maintenance/BIBS_CR_BRD-11_Change_Request_Register_v1.1.xlsx
+++ b/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-11_User_Access_Maintenance/BIBS_CR_BRD-11_Change_Request_Register_v1.1.xlsx
@@ -1202,7 +1202,7 @@
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>Already in BIBS?</t>
+          <t>Prepared for BIBS?</t>
         </is>
       </c>
       <c r="C12" s="14" t="inlineStr">
@@ -2052,7 +2052,7 @@
       </c>
       <c r="D4" s="24" t="inlineStr">
         <is>
-          <t>Already in BIBS?</t>
+          <t>Prepared for BIBS?</t>
         </is>
       </c>
       <c r="E4" s="24" t="inlineStr">

</xml_diff>

<commit_message>
BRD-11 BDOI-template FRS v1.4 rebuilt: three sources only (no BIBS build content), 64 full-page DEV screenshots one per page, BDOI UIDM review comments as integration scope (Annex Q.6, IS-UA-06 to 09), Annex AC User Access Report
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W3DAuLtsQmip7EuxjJCCtN
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-11_User_Access_Maintenance/BIBS_CR_BRD-11_Change_Request_Register_v1.1.xlsx
+++ b/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-11_User_Access_Maintenance/BIBS_CR_BRD-11_Change_Request_Register_v1.1.xlsx
@@ -24,7 +24,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Register'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Impact assessment form'!$A$12:$C$25</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Impact assessment form'!$12:$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Decisions log'!$A$4:$J$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Decisions log'!$A$4:$J$88</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Decisions log'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Lists'!$1:$1</definedName>
   </definedNames>
@@ -973,7 +973,7 @@
         </is>
       </c>
       <c r="D24" s="12" t="n">
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="26">
@@ -3305,7 +3305,7 @@
       </c>
       <c r="J15" s="12" t="inlineStr">
         <is>
-          <t>Only the time-based part is beyond the BRD: a number of working days per approval stage, a reminder to the approver before the limit and the escalation of an overdue request to the Business Administrator. The monitoring of the pending requests (configurable workflow, systematically monitored) is the BRD (NFR 11) and is a BRD item to deliver (BRD-UA-21); the escalation of out-of-hours and low-to-high privilege changes is BRD-UA-12.</t>
+          <t>Only the time-based part is beyond the BRD: a number of working days per approval stage, a reminder to the approver before the limit and the escalation of an overdue request to the Business Administrator. The monitoring of the pending requests (configurable workflow, systematically monitored) is the BRD (NFR 11) and is a BRD item to deliver for the requests that stay in the system (group-profile requests), the monitoring of the user access requests is done in UIDM-ISC (IS-UA-09, BDOI's review comments); the escalation of out-of-hours and low-to-high privilege changes is BRD-UA-12.</t>
         </is>
       </c>
       <c r="K15" s="12" t="inlineStr">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="S17" s="12" t="inlineStr">
         <is>
-          <t>Not a change request (review of 11-Oct-2026): Already a BRD requirement: UAM BRD Other BU NFR 10 "With Notification for access changes" and BRD 1.006.1.1, 1.008.1.4, 2.002.1 (receive notification on the returned, approved / rejected and to-approve request); the e-mail copy is a channel of those notifications (BRD-UA-20, Annex AA.4).</t>
+          <t>Not a change request (review of 11-Oct-2026): Already a BRD requirement: UAM BRD Other BU NFR 10 "With Notification for access changes" and BRD 1.006.1.1, 1.008.1.4, 2.002.1 (receive notification on the returned, approved / rejected and to-approve request); the e-mail copy is a channel of those notifications. With the request lifecycle in UIDM-ISC (BDOI's review comments, Annex Q.6) these notices and e-mails are sent by UIDM-ISC (IS-UA-09, Annex AA.5).</t>
         </is>
       </c>
       <c r="T17" s="12" t="inlineStr">
@@ -3841,7 +3841,7 @@
       </c>
       <c r="I20" s="12" t="inlineStr">
         <is>
-          <t>Emergency role edit: The emergency role edit setting, opened by Information Security; the direct edit of users and group profiles by the System Administrator while it is open, closed as delivered; every edit audited and alerted to Information Security; the marker on the screens.</t>
+          <t>Emergency role edit: The emergency role edit setting, opened by Information Security; the direct edit of users and group profiles by the System Administrator while it is open, closed by default; every edit audited and alerted to Information Security; the marker on the screens.</t>
         </is>
       </c>
       <c r="J20" s="12" t="inlineStr">
@@ -4259,7 +4259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J81"/>
+  <dimension ref="A1:J88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4370,7 +4370,7 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Option (a): UIDM-ISC provisions the user accounts (create, deactivate, reactivate) through the standard provisioning interface, each change logged with its UIDM request number; the assignment and change of group profiles and the group-profile requests stay as requests in the system under four eyes. FRUM.009 to FRUM.011 then apply to the changes not requested in UIDM; all of them apply if BDOI keeps every request in the system. Proposed behaviour: FRUM.009.01 to FRUM.009.10 and FRUM.010.01 to FRUM.010.05: every access change is a request in the system, decided by a chosen approver under four eyes; the UIDM-ISC option is open (CLR-UA-03). Available in BIBS: user accounts are created, updated, deactivated and reactivated from the Enterprise SSO and UIDM-ISC events (setting on by default, BDOI's text) or only through approved requests; the group profiles named in a UIDM-ISC event are applied only when a second setting is on (default off, option a).</t>
+          <t>Option (a): UIDM-ISC provisions the user accounts (create, deactivate, reactivate) through the standard provisioning interface, each change logged with its UIDM request number; the assignment and change of group profiles and the group-profile requests stay as requests in the system under four eyes. FRUM.009 to FRUM.011 then apply to the changes not requested in UIDM; all of them apply if BDOI keeps every request in the system. Proposed behaviour: FRUM.009.01 to FRUM.009.10 and FRUM.010.01 to FRUM.010.05: every access change is a request in the system, decided by a chosen approver under four eyes; the UIDM-ISC option is open (CLR-UA-03). Proposed (setting): user accounts are created, updated, deactivated and reactivated from the Enterprise SSO and UIDM-ISC events (setting on by default, BDOI's text) or only through approved requests; the group profiles named in a UIDM-ISC event are applied only when a second setting is on (default off, option a).</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -4478,7 +4478,7 @@
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>Create the user from the UIDM-ISC provisioning (which carries the SSO account) or from an approved enrolment; the Windows ID is checked against EIAM at the first sign-in. A look-up of the SSO directory on the enrolment screen is a change to the system for BDOI to decide. Proposed behaviour: FRUM.001.02, FRUM.001.06, FRUM.002.01, FRUM.009.02: the system never creates a user from a sign-in; the EIAM identity is linked to an existing active user by the Windows ID or the UPN (CLR-UA-22); the user is created by an approved enrolment or, as proposed, by UIDM-ISC provisioning. Available in BIBS: the user is created from an active Enterprise SSO account when the provisioning setting is on (default).</t>
+          <t>Create the user from the UIDM-ISC provisioning (which carries the SSO account) or from an approved enrolment; the Windows ID is checked against EIAM at the first sign-in. A look-up of the SSO directory on the enrolment screen is a change to the system for BDOI to decide. Proposed behaviour: FRUM.001.02, FRUM.001.06, FRUM.002.01, FRUM.009.02: the system never creates a user from a sign-in; the EIAM identity is linked to an existing active user by the Windows ID or the UPN (CLR-UA-22); the user is created by an approved enrolment or, as proposed, by UIDM-ISC provisioning. Proposed (setting): the user is created from an active Enterprise SSO account when the provisioning setting is on (default).</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
@@ -4586,7 +4586,7 @@
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Keep both - BDOI's message and Log In button after the inactivity sign-out (adopt the wording), and the warning before the fixed end of the session that the BRD asks. Proposed behaviour: FRUM.001.01, FRUM.001.03: sign-out after 30 minutes of inactivity with the warning at 15 minutes; a separate warning 30 minutes before the fixed end of the session. Available in BIBS: after the inactivity sign-out the page 'Your session timed out' with Log In is shown (setting on by default, BDOI's text) or a message on the Login page.</t>
+          <t>Keep both - BDOI's message and Log In button after the inactivity sign-out (adopt the wording), and the warning before the fixed end of the session that the BRD asks. Proposed behaviour: FRUM.001.01, FRUM.001.03: sign-out after 30 minutes of inactivity with the warning at 15 minutes; a separate warning 30 minutes before the fixed end of the session. Proposed (setting): after the inactivity sign-out the page 'Your session timed out' with Log In is shown (setting on by default, BDOI's text) or a message on the Login page.</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
@@ -4622,7 +4622,7 @@
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
-          <t>Adopt BDOI's text and buttons (a screen text change, no rule change). Proposed behaviour: FRUM.001.01, FRUM.001.03 and the session dialog of the screens: "For your security the system signs you out in n minute(s)..." with the system's own buttons. Available in BIBS: the inactivity warning uses BDOI's wording and the buttons Stay Logged In and Log Out (setting on by default) or the earlier wording.</t>
+          <t>Adopt BDOI's text and buttons (a screen text change, no rule change). Proposed behaviour: FRUM.001.01, FRUM.001.03 and the session dialog of the screens: "For your security the system signs you out in n minute(s)..." with the system's own buttons. Proposed (setting): the inactivity warning uses BDOI's wording and the buttons Stay Logged In and Log Out (setting on by default) or the earlier wording.</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -4694,7 +4694,7 @@
       </c>
       <c r="D14" s="12" t="inlineStr">
         <is>
-          <t>Adopt 10 for the local accounts (a setting value, no change). Proposed behaviour: FRUM-004.01, FRUM-004.02: history of 8 for local accounts (value to confirm, UQ08). Available in BIBS: the number of previous passwords that may not be reused is a security setting, delivered at 10 (BDOI's text).</t>
+          <t>Adopt 10 for the local accounts (a setting value, no change). Proposed behaviour: FRUM-004.01, FRUM-004.02: history of 8 for local accounts (value to confirm, UQ08). Proposed (setting): the number of previous passwords that may not be reused is a security setting, delivered at 10 (BDOI's text).</t>
         </is>
       </c>
       <c r="E14" s="12" t="inlineStr">
@@ -4730,7 +4730,7 @@
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>SSO users: BDOI's rule (no reset in the application). Break-glass accounts: reset by a second administrator only; the self-service link switched off in production. Proposed behaviour: FRUM-004.01, FRUM-004.02: for local accounts, an administrator reset and a self-service reset link; none for SSO users. Available in BIBS: no forgotten-password link and reset by another System Administrator only (setting on by default, BDOI's text) or the self-service reset of local accounts.</t>
+          <t>SSO users: BDOI's rule (no reset in the application). Break-glass accounts: reset by a second administrator only; the self-service link switched off in production. Proposed behaviour: FRUM-004.01, FRUM-004.02: for local accounts, an administrator reset and a self-service reset link; none for SSO users. Proposed (setting): no forgotten-password link and reset by another System Administrator only (setting on by default, BDOI's text) or the self-service reset of local accounts.</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
@@ -4802,7 +4802,7 @@
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>With option (a), a leaver from UIDM-ISC deactivates the user and ends the open sessions at once (change to the system); a deactivation request does the same on approval. Proposed behaviour: FRUM.003.02.01, FRUM.009.04, FRUM.003.02.01, FRUM.003.04: deactivation by a request or the dormant-user job; EIAM refuses a disabled BDO account at the next sign-in; the open session ends at the inactivity sign-out or the session expiry. Available in BIBS: access is revoked and restored from the Enterprise SSO status when the provisioning setting is on (default).</t>
+          <t>With option (a), a leaver from UIDM-ISC deactivates the user and ends the open sessions at once (change to the system); a deactivation request does the same on approval. Proposed behaviour: FRUM.003.02.01, FRUM.009.04, FRUM.003.02.01, FRUM.003.04: deactivation by a request or the dormant-user job; EIAM refuses a disabled BDO account at the next sign-in; the open session ends at the inactivity sign-out or the session expiry. Proposed (setting): access is revoked and restored from the Enterprise SSO status when the provisioning setting is on (default).</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
@@ -4838,7 +4838,7 @@
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>Show on each user the last provisioning event (time, source, UIDM request number); refuse a failed provisioning call back to UIDM-ISC and alert the System Administrator; replace the on-demand synchronisation by a re-send from UIDM-ISC. Proposed behaviour: None; the UIDM-ISC option (a) pushes changes to the system; the Users screen shows the last sign-in. Available in BIBS: synchronisation from the Enterprise SSO runs on each event and on demand when the provisioning setting is on (default).</t>
+          <t>Show on each user the last provisioning event (time, source, UIDM request number); refuse a failed provisioning call back to UIDM-ISC and alert the System Administrator; replace the on-demand synchronisation by a re-send from UIDM-ISC. Proposed behaviour: None; the UIDM-ISC option (a) pushes changes to the system; the Users screen shows the last sign-in. Proposed (setting): synchronisation from the Enterprise SSO runs on each event and on demand when the provisioning setting is on (default).</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
@@ -4910,7 +4910,7 @@
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>Keep the rules at group-profile level (what one user may hold); BDOI lists the permission pairs it means and they become rules between profiles. Proposed behaviour: FRUM.006.03, FRUM.012.01: separation-of-duties rules name pairs of group profiles one user may not hold, maintained by the Business Administrator and authorised by Information Security; FRUM.006.01, FRUM.006.03 refuses a permission both added and removed. Available in BIBS: the conflicting permission combinations are rules maintained by Information Security under a second approval.</t>
+          <t>Keep the rules at group-profile level (what one user may hold); BDOI lists the permission pairs it means and they become rules between profiles. Proposed behaviour: FRUM.006.03, FRUM.012.01: separation-of-duties rules name pairs of group profiles one user may not hold, maintained by the Business Administrator and authorised by Information Security; FRUM.006.01, FRUM.006.03 refuses a permission both added and removed. Proposed (setting): the conflicting permission combinations are rules maintained by Information Security under a second approval.</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
@@ -4982,7 +4982,7 @@
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>Adopt BDOI's file names (a change of the download name). Proposed behaviour: FRUM.007.01, FRUM.007.02 to FRUM.008.01, FRUM.008.01 (2nd): report name, generated by, coverage and time generated in the header; the file name is not specified. Available in BIBS: the exports are named by BDOI's convention &lt;name&gt;_MMDDYYYY (setting on by default) or by the report code.</t>
+          <t>Adopt BDOI's file names (a change of the download name). Proposed behaviour: FRUM.007.01, FRUM.007.02 to FRUM.008.01, FRUM.008.01 (2nd): report name, generated by, coverage and time generated in the header; the file name is not specified. Proposed (setting): the exports are named by BDOI's convention &lt;name&gt;_MMDDYYYY (setting on by default) or by the report code.</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
@@ -5234,7 +5234,7 @@
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>Add as FRUM.013.01. Proposed behaviour: FRUM.013.01: notices to the approver, the requester and the affected user, in the system and by e-mail. Available in BIBS: the notices of access requests are also e-mailed by each user's notification preference (setting on by default) or shown in the system only.</t>
+          <t>Add as FRUM.013.01. Proposed behaviour: FRUM.013.01: notices to the approver, the requester and the affected user, in the system and by e-mail. Proposed (setting): the notices of access requests are also e-mailed by each user's notification preference (setting on by default) or shown in the system only.</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
@@ -7124,23 +7124,275 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" s="12" t="inlineStr">
+        <is>
+          <t>Q-78</t>
+        </is>
+      </c>
+      <c r="B82" s="12" t="inlineStr">
+        <is>
+          <t>Q.6</t>
+        </is>
+      </c>
+      <c r="C82" s="12" t="inlineStr">
+        <is>
+          <t>Review comment on BRD 1.006.1 – Apply correction on returned requests</t>
+        </is>
+      </c>
+      <c r="D82" s="12" t="inlineStr">
+        <is>
+          <t>Agreed: the correction of a returned request is done in UIDM-ISC ("c/o UIDM"). FRUM.009.07 is labelled [Integration scope – UIDM-ISC] and listed in Annex AA.5 (IS-UA-06); the system receives the corrected and approved change through the provisioning interface (Annex N.3). Its delivery effort is removed from the BRD items to deliver.</t>
+        </is>
+      </c>
+      <c r="E82" s="12" t="inlineStr">
+        <is>
+          <t>BDOI (comment author)</t>
+        </is>
+      </c>
+      <c r="F82" s="12" t="inlineStr"/>
+      <c r="G82" s="12" t="inlineStr"/>
+      <c r="H82" s="12" t="inlineStr"/>
+      <c r="I82" s="12" t="inlineStr"/>
+      <c r="J82" s="25" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="12" t="inlineStr">
+        <is>
+          <t>Q-79</t>
+        </is>
+      </c>
+      <c r="B83" s="12" t="inlineStr">
+        <is>
+          <t>Q.6</t>
+        </is>
+      </c>
+      <c r="C83" s="12" t="inlineStr">
+        <is>
+          <t>Review comment on BRD 1.007.1 – Cancel a submitted request</t>
+        </is>
+      </c>
+      <c r="D83" s="12" t="inlineStr">
+        <is>
+          <t>Agreed: a submitted request is cancelled in UIDM-ISC. FRUM.009.08 is labelled [Integration scope – UIDM-ISC] (Annex AA.5, IS-UA-06); nothing reaches the system for a cancelled request.</t>
+        </is>
+      </c>
+      <c r="E83" s="12" t="inlineStr">
+        <is>
+          <t>BDOI (comment author)</t>
+        </is>
+      </c>
+      <c r="F83" s="12" t="inlineStr"/>
+      <c r="G83" s="12" t="inlineStr"/>
+      <c r="H83" s="12" t="inlineStr"/>
+      <c r="I83" s="12" t="inlineStr"/>
+      <c r="J83" s="25" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="12" t="inlineStr">
+        <is>
+          <t>Q-80</t>
+        </is>
+      </c>
+      <c r="B84" s="12" t="inlineStr">
+        <is>
+          <t>Q.6</t>
+        </is>
+      </c>
+      <c r="C84" s="12" t="inlineStr">
+        <is>
+          <t>Review comment on BRD 1.008.1 – View the submitted requests</t>
+        </is>
+      </c>
+      <c r="D84" s="12" t="inlineStr">
+        <is>
+          <t>Agreed: the requester follows the submitted requests in UIDM-ISC. FRUM.009.09 is labelled [Integration scope – UIDM-ISC] (Annex AA.5, IS-UA-06); the system keeps the UIDM request number on every change it applies, so the reports of FRUM.007 and FRUM.008 still show it.</t>
+        </is>
+      </c>
+      <c r="E84" s="12" t="inlineStr">
+        <is>
+          <t>BDOI (comment author)</t>
+        </is>
+      </c>
+      <c r="F84" s="12" t="inlineStr"/>
+      <c r="G84" s="12" t="inlineStr"/>
+      <c r="H84" s="12" t="inlineStr"/>
+      <c r="I84" s="12" t="inlineStr"/>
+      <c r="J84" s="25" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="12" t="inlineStr">
+        <is>
+          <t>Q-81</t>
+        </is>
+      </c>
+      <c r="B85" s="12" t="inlineStr">
+        <is>
+          <t>Q.6</t>
+        </is>
+      </c>
+      <c r="C85" s="12" t="inlineStr">
+        <is>
+          <t>Review comment on BRD 1.009.1 – Bulk request</t>
+        </is>
+      </c>
+      <c r="D85" s="12" t="inlineStr">
+        <is>
+          <t>Agreed: bulk requests are raised and approved in UIDM-ISC. FRUM.011.01 is labelled [Integration scope – UIDM-ISC] (Annex AA.5, IS-UA-07); the loading of the users at go-live stays data migration (DM-UA-01).</t>
+        </is>
+      </c>
+      <c r="E85" s="12" t="inlineStr">
+        <is>
+          <t>BDOI (comment author)</t>
+        </is>
+      </c>
+      <c r="F85" s="12" t="inlineStr"/>
+      <c r="G85" s="12" t="inlineStr"/>
+      <c r="H85" s="12" t="inlineStr"/>
+      <c r="I85" s="12" t="inlineStr"/>
+      <c r="J85" s="25" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="12" t="inlineStr">
+        <is>
+          <t>Q-82</t>
+        </is>
+      </c>
+      <c r="B86" s="12" t="inlineStr">
+        <is>
+          <t>Q.6</t>
+        </is>
+      </c>
+      <c r="C86" s="12" t="inlineStr">
+        <is>
+          <t>Review comment on BRD 2.002.1 – Review and approve requests (receive, list, approve, reject, return)</t>
+        </is>
+      </c>
+      <c r="D86" s="12" t="inlineStr">
+        <is>
+          <t>Agreed: the approver reviews, approves, rejects and returns the user access requests in UIDM-ISC, with the notices of each step. FRUM.010.01 to FRUM.010.05 are labelled [Integration scope – UIDM-ISC] (Annex AA.5, IS-UA-08 and IS-UA-09). The group-profile requests of BRD 3.002 (FRUM.005, FRUM.006, FRUM.011 group profiles) have no such comment and stay in the system; if BDOI keeps the assignment of group profiles as requests in the system (option (a) of Annex N.3), the approval of those requests also stays in the system (Q-01).</t>
+        </is>
+      </c>
+      <c r="E86" s="12" t="inlineStr">
+        <is>
+          <t>BDOI (comment author)</t>
+        </is>
+      </c>
+      <c r="F86" s="12" t="inlineStr"/>
+      <c r="G86" s="12" t="inlineStr"/>
+      <c r="H86" s="12" t="inlineStr"/>
+      <c r="I86" s="12" t="inlineStr"/>
+      <c r="J86" s="25" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="12" t="inlineStr">
+        <is>
+          <t>Q-83</t>
+        </is>
+      </c>
+      <c r="B87" s="12" t="inlineStr">
+        <is>
+          <t>Q.6</t>
+        </is>
+      </c>
+      <c r="C87" s="12" t="inlineStr">
+        <is>
+          <t>Review comment on BRD 3.003.1.1 – User Access Report fields</t>
+        </is>
+      </c>
+      <c r="D87" s="12" t="inlineStr">
+        <is>
+          <t>Added: Annex AC gives the User Access Report fields of BRD 3.003.1 and Annex E with a sample layout. The sample sent in Ruby's e-mail will replace it once received: Ruby's e-mail address and the sample are an open question to BDOI (Q.6, last row); the address is not assumed.</t>
+        </is>
+      </c>
+      <c r="E87" s="12" t="inlineStr">
+        <is>
+          <t>BDOI (comment author)</t>
+        </is>
+      </c>
+      <c r="F87" s="12" t="inlineStr"/>
+      <c r="G87" s="12" t="inlineStr"/>
+      <c r="H87" s="12" t="inlineStr"/>
+      <c r="I87" s="12" t="inlineStr"/>
+      <c r="J87" s="25" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="12" t="inlineStr">
+        <is>
+          <t>Q-84</t>
+        </is>
+      </c>
+      <c r="B88" s="12" t="inlineStr">
+        <is>
+          <t>Q.6</t>
+        </is>
+      </c>
+      <c r="C88" s="12" t="inlineStr">
+        <is>
+          <t>User Access Report sample from Ruby's e-mail</t>
+        </is>
+      </c>
+      <c r="D88" s="12" t="inlineStr">
+        <is>
+          <t>BDOI to give Ruby's e-mail address (and Ruby's full name and unit) and to forward the e-mail with the User Access Report sample; Annex AC is then updated to the sample. Until then Annex AC shows the layout of BRD 3.003.1 and Annex E.</t>
+        </is>
+      </c>
+      <c r="E88" s="12" t="inlineStr">
+        <is>
+          <t>John V. Barbachano (BDO ITG); Process Owner (Business Administration)</t>
+        </is>
+      </c>
+      <c r="F88" s="12" t="inlineStr"/>
+      <c r="G88" s="12" t="inlineStr"/>
+      <c r="H88" s="12" t="inlineStr"/>
+      <c r="I88" s="12" t="inlineStr"/>
+      <c r="J88" s="25" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:J81"/>
+  <autoFilter ref="A4:J88"/>
   <mergeCells count="1">
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="J5:J581">
+  <conditionalFormatting sqref="J5:J588">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="2" stopIfTrue="1">
       <formula>"Open"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:J581">
+  <conditionalFormatting sqref="A5:J588">
     <cfRule type="expression" priority="2" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="J5:J581" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
+    <dataValidation sqref="J5:J588" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
       <formula1>'Lists'!$D$2:$D$4</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>